<commit_message>
fix issue with kevin's number code in the excel file. Was duplicate of 80. Added 81.
</commit_message>
<xml_diff>
--- a/python-notebooks/billing.xlsx
+++ b/python-notebooks/billing.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/klowe/repos-personal/energy-project/python-notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A28A1B-34C6-7F47-AE7E-CDA7A7073F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313C4873-0570-0147-BAB6-D67ED3061733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -402,11 +402,6 @@
 (35)</t>
   </si>
   <si>
-    <t xml:space="preserve"> PCE Generation Charges due in Cash 
-[$]
-(80)</t>
-  </si>
-  <si>
     <t>allocation 
 [%]</t>
   </si>
@@ -414,6 +409,11 @@
     <t>NEM True Up Adjustment
 [$]
 (80)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> PCE Generation Charges due in Cash 
+[$]
+(81)</t>
   </si>
 </sst>
 </file>
@@ -1562,7 +1562,7 @@
         <v>64</v>
       </c>
       <c r="AA6" s="51" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AB6" s="51" t="s">
         <v>65</v>
@@ -1583,7 +1583,7 @@
         <v>70</v>
       </c>
       <c r="AH6" s="51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AI6" s="51" t="s">
         <v>71</v>
@@ -1613,7 +1613,7 @@
         <v>76</v>
       </c>
       <c r="AR6" s="51" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AS6" s="51" t="s">
         <v>77</v>
@@ -1795,11 +1795,11 @@
         <v>395</v>
       </c>
       <c r="AO7" s="15">
-        <f>D7-J7</f>
+        <f t="shared" ref="AO7:AP11" si="6">D7-J7</f>
         <v>-449</v>
       </c>
       <c r="AP7" s="15">
-        <f>E7-K7</f>
+        <f t="shared" si="6"/>
         <v>-58</v>
       </c>
       <c r="AQ7" s="15">
@@ -1828,7 +1828,7 @@
         <v>5.8379099999999999</v>
       </c>
       <c r="AX7" s="17">
-        <f t="shared" ref="AX7:AX8" si="6">AW7+AV7</f>
+        <f t="shared" ref="AX7:AX8" si="7">AW7+AV7</f>
         <v>-13.174499999999998</v>
       </c>
       <c r="AY7" s="17">
@@ -1868,7 +1868,7 @@
         <v>45456</v>
       </c>
       <c r="D8" s="15">
-        <f t="shared" ref="D8" si="7">ROUND(J8/M8,0)</f>
+        <f t="shared" ref="D8" si="8">ROUND(J8/M8,0)</f>
         <v>-1411</v>
       </c>
       <c r="E8" s="15">
@@ -1879,11 +1879,11 @@
         <v>-1601</v>
       </c>
       <c r="G8" s="15">
-        <f t="shared" ref="G8:H8" si="8">G9+G10</f>
+        <f t="shared" ref="G8:H8" si="9">G9+G10</f>
         <v>330</v>
       </c>
       <c r="H8" s="15">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>121</v>
       </c>
       <c r="I8" s="15">
@@ -1905,23 +1905,23 @@
         <v>0.49906308557151779</v>
       </c>
       <c r="N8" s="15">
-        <f t="shared" ref="N8:R8" si="9">N9+N10</f>
+        <f t="shared" ref="N8:R8" si="10">N9+N10</f>
         <v>-374</v>
       </c>
       <c r="O8" s="15">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>26</v>
       </c>
       <c r="P8" s="15">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-348</v>
       </c>
       <c r="Q8" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>-47.806659999999994</v>
       </c>
       <c r="R8" s="17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.8457699999999995</v>
       </c>
       <c r="S8" s="17">
@@ -1980,7 +1980,7 @@
         <v>0</v>
       </c>
       <c r="AI8" s="17">
-        <f t="shared" ref="AI8" si="10">AF8+AG8+AH8</f>
+        <f t="shared" ref="AI8" si="11">AF8+AG8+AH8</f>
         <v>21.75</v>
       </c>
       <c r="AJ8" s="15">
@@ -1991,22 +1991,22 @@
         <v>21.75</v>
       </c>
       <c r="AL8" s="15">
-        <f t="shared" ref="AL8:AM8" si="11">AS8-AO8</f>
+        <f t="shared" ref="AL8:AM8" si="12">AS8-AO8</f>
         <v>349</v>
       </c>
       <c r="AM8" s="15">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>102</v>
       </c>
       <c r="AN8" s="15">
         <v>451</v>
       </c>
       <c r="AO8" s="15">
-        <f>D8-J8</f>
+        <f t="shared" si="6"/>
         <v>-707</v>
       </c>
       <c r="AP8" s="15">
-        <f>E8-K8</f>
+        <f t="shared" si="6"/>
         <v>-95</v>
       </c>
       <c r="AQ8" s="15">
@@ -2021,23 +2021,23 @@
         <v>-358</v>
       </c>
       <c r="AT8" s="15">
-        <f t="shared" ref="AT8:AW8" si="12">AT9+AT10</f>
+        <f t="shared" ref="AT8:AW8" si="13">AT9+AT10</f>
         <v>7</v>
       </c>
       <c r="AU8" s="15">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-351</v>
       </c>
       <c r="AV8" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>-45.9373</v>
       </c>
       <c r="AW8" s="17">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.77081</v>
       </c>
       <c r="AX8" s="17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-45.166490000000003</v>
       </c>
       <c r="AY8" s="17">
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="BA8" s="20">
-        <f t="shared" ref="BA7:BA8" si="13">AZ8+AY8+AX8</f>
+        <f t="shared" ref="BA8" si="14">AZ8+AY8+AX8</f>
         <v>-48.806490000000004</v>
       </c>
       <c r="BB8" s="21">
@@ -2064,7 +2064,7 @@
         <v>0</v>
       </c>
       <c r="BF8" s="22">
-        <f t="shared" ref="BF8" si="14">BD8+BC8+BE8</f>
+        <f t="shared" ref="BF8" si="15">BD8+BC8+BE8</f>
         <v>11.75</v>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
         <v>27</v>
       </c>
       <c r="P9" s="25">
-        <f t="shared" ref="P9:P11" si="15">O9+N9</f>
+        <f t="shared" ref="P9:P11" si="16">O9+N9</f>
         <v>-273</v>
       </c>
       <c r="Q9" s="27">
@@ -2145,11 +2145,11 @@
       </c>
       <c r="AN9" s="58"/>
       <c r="AO9" s="58">
-        <f>D9-J9</f>
+        <f t="shared" si="6"/>
         <v>-575</v>
       </c>
       <c r="AP9" s="58">
-        <f>E9-K9</f>
+        <f t="shared" si="6"/>
         <v>-77</v>
       </c>
       <c r="AQ9" s="25"/>
@@ -2161,7 +2161,7 @@
         <v>13</v>
       </c>
       <c r="AU9" s="25">
-        <f t="shared" ref="AU9:AU11" si="16">AT9+AS9</f>
+        <f t="shared" ref="AU9:AU11" si="17">AT9+AS9</f>
         <v>-256</v>
       </c>
       <c r="AV9" s="27">
@@ -2219,15 +2219,15 @@
         <v>-1</v>
       </c>
       <c r="P10" s="25">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-75</v>
       </c>
       <c r="Q10" s="27">
-        <f t="shared" ref="Q10:Q11" si="17">N10*0.13559</f>
+        <f t="shared" ref="Q10:Q11" si="18">N10*0.13559</f>
         <v>-10.033659999999999</v>
       </c>
       <c r="R10" s="27">
-        <f t="shared" ref="R10:R11" si="18">O10*0.19586</f>
+        <f t="shared" ref="R10:R11" si="19">O10*0.19586</f>
         <v>-0.19586000000000001</v>
       </c>
       <c r="S10" s="27"/>
@@ -2259,11 +2259,11 @@
       </c>
       <c r="AN10" s="58"/>
       <c r="AO10" s="58">
-        <f>D10-J10</f>
+        <f t="shared" si="6"/>
         <v>-131</v>
       </c>
       <c r="AP10" s="58">
-        <f>E10-K10</f>
+        <f t="shared" si="6"/>
         <v>-18</v>
       </c>
       <c r="AQ10" s="25"/>
@@ -2275,15 +2275,15 @@
         <v>-6</v>
       </c>
       <c r="AU10" s="25">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>-95</v>
       </c>
       <c r="AV10" s="27">
-        <f t="shared" ref="AV10:AV11" si="19">AS10*0.13559</f>
+        <f t="shared" ref="AV10:AV11" si="20">AS10*0.13559</f>
         <v>-12.067509999999999</v>
       </c>
       <c r="AW10" s="27">
-        <f t="shared" ref="AW10:AW11" si="20">AT10*0.19586</f>
+        <f t="shared" ref="AW10:AW11" si="21">AT10*0.19586</f>
         <v>-1.17516</v>
       </c>
       <c r="AX10" s="27"/>
@@ -2316,11 +2316,11 @@
         <v>-1750</v>
       </c>
       <c r="G11" s="15">
-        <f t="shared" ref="G11:H11" si="21">G12+G13</f>
+        <f t="shared" ref="G11:H11" si="22">G12+G13</f>
         <v>393</v>
       </c>
       <c r="H11" s="15">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>250</v>
       </c>
       <c r="I11" s="15">
@@ -2331,7 +2331,7 @@
         <v>-1001</v>
       </c>
       <c r="K11" s="15">
-        <f t="shared" ref="K11" si="22">K12+K13</f>
+        <f t="shared" ref="K11" si="23">K12+K13</f>
         <v>-131</v>
       </c>
       <c r="L11" s="15">
@@ -2348,15 +2348,15 @@
         <v>119</v>
       </c>
       <c r="P11" s="15">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>-489</v>
       </c>
       <c r="Q11" s="17">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-82.438719999999989</v>
       </c>
       <c r="R11" s="17">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>23.30734</v>
       </c>
       <c r="S11" s="17">
@@ -2426,22 +2426,22 @@
         <v>22.53</v>
       </c>
       <c r="AL11" s="15">
-        <f t="shared" ref="AL11:AM11" si="23">AS11-AO11</f>
+        <f t="shared" ref="AL11:AM11" si="24">AS11-AO11</f>
         <v>276</v>
       </c>
       <c r="AM11" s="15">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>53</v>
       </c>
       <c r="AN11" s="15">
         <v>329</v>
       </c>
       <c r="AO11" s="15">
-        <f>D11-J11</f>
+        <f t="shared" si="6"/>
         <v>-546</v>
       </c>
       <c r="AP11" s="15">
-        <f>E11-K11</f>
+        <f t="shared" si="6"/>
         <v>-72</v>
       </c>
       <c r="AQ11" s="15">
@@ -2458,15 +2458,15 @@
         <v>-19</v>
       </c>
       <c r="AU11" s="15">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>-289</v>
       </c>
       <c r="AV11" s="17">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>-36.609299999999998</v>
       </c>
       <c r="AW11" s="17">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>-3.7213400000000001</v>
       </c>
       <c r="AX11" s="17">
@@ -2695,23 +2695,23 @@
         <v>0.40445402298850575</v>
       </c>
       <c r="N14" s="33">
-        <f t="shared" ref="N14:P14" si="24">N15+N16</f>
+        <f t="shared" ref="N14:P14" si="25">N15+N16</f>
         <v>-267</v>
       </c>
       <c r="O14" s="33">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>86</v>
       </c>
       <c r="P14" s="34">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>-181</v>
       </c>
       <c r="Q14" s="17">
-        <f t="shared" ref="Q14:R14" si="25">SUM(Q15:Q16)</f>
+        <f t="shared" ref="Q14:R14" si="26">SUM(Q15:Q16)</f>
         <v>-35.405396597999996</v>
       </c>
       <c r="R14" s="17">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>16.917801365000003</v>
       </c>
       <c r="S14" s="17">
@@ -2781,11 +2781,11 @@
         <v>21.36</v>
       </c>
       <c r="AL14" s="15">
-        <f t="shared" ref="AL14:AM14" si="26">AS14-AO14</f>
+        <f t="shared" ref="AL14:AM14" si="27">AS14-AO14</f>
         <v>409</v>
       </c>
       <c r="AM14" s="15">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>132</v>
       </c>
       <c r="AN14" s="15">
@@ -2807,23 +2807,23 @@
         <v>0.59554597701149425</v>
       </c>
       <c r="AS14" s="15">
-        <f t="shared" ref="AS14:AU14" si="27">AS15+AS16</f>
+        <f t="shared" ref="AS14:AU14" si="28">AS15+AS16</f>
         <v>-314</v>
       </c>
       <c r="AT14" s="15">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>26</v>
       </c>
       <c r="AU14" s="15">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>-288</v>
       </c>
       <c r="AV14" s="17">
-        <f t="shared" ref="AV14:AW14" si="28">SUM(AV15:AV16)</f>
+        <f t="shared" ref="AV14:AW14" si="29">SUM(AV15:AV16)</f>
         <v>-41.637807834999997</v>
       </c>
       <c r="AW14" s="17">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>5.1146840949999994</v>
       </c>
       <c r="AX14" s="17">
@@ -2925,7 +2925,7 @@
         <v>20.620699999999999</v>
       </c>
       <c r="AU15" s="36">
-        <f t="shared" ref="AU15:AU17" si="29">AT15+AS15</f>
+        <f t="shared" ref="AU15:AU17" si="30">AT15+AS15</f>
         <v>-44.344800000000006</v>
       </c>
       <c r="AV15" s="39">
@@ -2977,7 +2977,7 @@
         <v>-28.712348573999996</v>
       </c>
       <c r="R16" s="39">
-        <f t="shared" ref="R16:R17" si="30">O16*0.20001</f>
+        <f t="shared" ref="R16:R17" si="31">O16*0.20001</f>
         <v>3.5587979309999995</v>
       </c>
       <c r="S16" s="39"/>
@@ -3013,7 +3013,7 @@
         <v>5.3792999999999997</v>
       </c>
       <c r="AU16" s="36">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>-243.65520000000001</v>
       </c>
       <c r="AV16" s="39">
@@ -3021,7 +3021,7 @@
         <v>-33.766587854999997</v>
       </c>
       <c r="AW16" s="39">
-        <f t="shared" ref="AW16:AW17" si="31">AT16*0.20001</f>
+        <f t="shared" ref="AW16:AW17" si="32">AT16*0.20001</f>
         <v>1.075913793</v>
       </c>
       <c r="AX16" s="39"/>
@@ -3054,11 +3054,11 @@
         <v>-1516</v>
       </c>
       <c r="G17" s="15">
-        <f t="shared" ref="G17:H17" si="32">G18+G19</f>
+        <f t="shared" ref="G17:H17" si="33">G18+G19</f>
         <v>175</v>
       </c>
       <c r="H17" s="15">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>145</v>
       </c>
       <c r="I17" s="15">
@@ -3069,7 +3069,7 @@
         <v>-386</v>
       </c>
       <c r="K17" s="15">
-        <f t="shared" ref="K17" si="33">K18+K19</f>
+        <f t="shared" ref="K17" si="34">K18+K19</f>
         <v>-50</v>
       </c>
       <c r="L17" s="15">
@@ -3094,7 +3094,7 @@
         <v>-25.56476</v>
       </c>
       <c r="R17" s="17">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>19.00095</v>
       </c>
       <c r="S17" s="17">
@@ -3164,11 +3164,11 @@
         <v>21.75</v>
       </c>
       <c r="AL17" s="15">
-        <f t="shared" ref="AL17:AM17" si="34">AS17-AO17</f>
+        <f t="shared" ref="AL17:AM17" si="35">AS17-AO17</f>
         <v>519</v>
       </c>
       <c r="AM17" s="15">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>203</v>
       </c>
       <c r="AN17" s="15">
@@ -3196,7 +3196,7 @@
         <v>80</v>
       </c>
       <c r="AU17" s="15">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>-354</v>
       </c>
       <c r="AV17" s="17">
@@ -3204,7 +3204,7 @@
         <v>-52.583440000000003</v>
       </c>
       <c r="AW17" s="17">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>16.000799999999998</v>
       </c>
       <c r="AX17" s="17">
@@ -3414,7 +3414,7 @@
         <v>69</v>
       </c>
       <c r="P20" s="69">
-        <f t="shared" ref="P20:P22" si="35">O20+N20</f>
+        <f t="shared" ref="P20:P22" si="36">O20+N20</f>
         <v>-76</v>
       </c>
       <c r="Q20" s="27">
@@ -3458,7 +3458,7 @@
         <v>99</v>
       </c>
       <c r="AU20" s="25">
-        <f t="shared" ref="AU20:AU22" si="36">AT20+AS20</f>
+        <f t="shared" ref="AU20:AU22" si="37">AT20+AS20</f>
         <v>-176</v>
       </c>
       <c r="AV20" s="27">
@@ -3502,7 +3502,7 @@
         <v>62</v>
       </c>
       <c r="P21" s="69">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>64</v>
       </c>
       <c r="Q21" s="27">
@@ -3546,7 +3546,7 @@
         <v>33</v>
       </c>
       <c r="AU21" s="25">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>-13</v>
       </c>
       <c r="AV21" s="27">
@@ -3587,22 +3587,22 @@
         <v>-1292</v>
       </c>
       <c r="G22" s="15">
-        <f t="shared" ref="G22:H22" si="37">G23+G24</f>
+        <f t="shared" ref="G22:H22" si="38">G23+G24</f>
         <v>191</v>
       </c>
       <c r="H22" s="15">
-        <f t="shared" si="37"/>
+        <f t="shared" si="38"/>
         <v>157</v>
       </c>
       <c r="I22" s="15">
         <v>348</v>
       </c>
       <c r="J22" s="15">
-        <f t="shared" ref="J22:K22" si="38">J23+J24</f>
+        <f t="shared" ref="J22:K22" si="39">J23+J24</f>
         <v>-334</v>
       </c>
       <c r="K22" s="15">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>-26</v>
       </c>
       <c r="L22" s="15">
@@ -3613,23 +3613,23 @@
         <v>0.27863777089783281</v>
       </c>
       <c r="N22" s="15">
-        <f t="shared" ref="N22:O22" si="39">N21+N20</f>
+        <f t="shared" ref="N22:O22" si="40">N21+N20</f>
         <v>-143</v>
       </c>
       <c r="O22" s="15">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>131</v>
       </c>
       <c r="P22" s="15">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>-12</v>
       </c>
       <c r="Q22" s="17">
-        <f t="shared" ref="Q22:R22" si="40">Q20+Q21</f>
+        <f t="shared" ref="Q22:R22" si="41">Q20+Q21</f>
         <v>-17.332979999999999</v>
       </c>
       <c r="R22" s="17">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>22.664209999999997</v>
       </c>
       <c r="S22" s="17">
@@ -3699,11 +3699,11 @@
         <v>-33.03</v>
       </c>
       <c r="AL22" s="15">
-        <f t="shared" ref="AL22:AM22" si="41">AS22-AO22</f>
+        <f t="shared" ref="AL22:AM22" si="42">AS22-AO22</f>
         <v>544</v>
       </c>
       <c r="AM22" s="15">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>199</v>
       </c>
       <c r="AN22" s="15">
@@ -3733,15 +3733,15 @@
         <v>132</v>
       </c>
       <c r="AU22" s="15">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v>-189</v>
       </c>
       <c r="AV22" s="17">
-        <f t="shared" ref="AV22:AW22" si="42">AV20+AV21</f>
+        <f t="shared" ref="AV22:AW22" si="43">AV20+AV21</f>
         <v>-38.729060000000004</v>
       </c>
       <c r="AW22" s="17">
-        <f t="shared" si="42"/>
+        <f t="shared" si="43"/>
         <v>24.51867</v>
       </c>
       <c r="AX22" s="17">
@@ -3772,7 +3772,7 @@
         <v>-55.17</v>
       </c>
       <c r="BF22" s="22">
-        <f t="shared" ref="BF22" si="43">BD22+BC22+BE22</f>
+        <f t="shared" ref="BF22" si="44">BD22+BC22+BE22</f>
         <v>-43.03</v>
       </c>
     </row>
@@ -3976,19 +3976,19 @@
         <v>191</v>
       </c>
       <c r="P25" s="43">
-        <f t="shared" ref="P25:P27" si="44">O25+N25</f>
+        <f t="shared" ref="P25:P27" si="45">O25+N25</f>
         <v>59</v>
       </c>
       <c r="Q25" s="45">
-        <f t="shared" ref="Q25:Q27" si="45">N25*0.11761</f>
+        <f t="shared" ref="Q25:Q27" si="46">N25*0.11761</f>
         <v>-15.524520000000001</v>
       </c>
       <c r="R25" s="45">
-        <f t="shared" ref="R25:R27" si="46">O25*0.14296</f>
+        <f t="shared" ref="R25:R27" si="47">O25*0.14296</f>
         <v>27.30536</v>
       </c>
       <c r="S25" s="45">
-        <f t="shared" ref="S25:S27" si="47">R25+Q25</f>
+        <f t="shared" ref="S25:S27" si="48">R25+Q25</f>
         <v>11.78084</v>
       </c>
       <c r="T25" s="45">
@@ -3996,15 +3996,15 @@
         <v>-1.32</v>
       </c>
       <c r="U25" s="18">
-        <f t="shared" ref="U25:U27" si="48">(ABS(Q25)+ABS(R25))/(ABS(N25)+ABS(O25))</f>
+        <f t="shared" ref="U25:U27" si="49">(ABS(Q25)+ABS(R25))/(ABS(N25)+ABS(O25))</f>
         <v>0.13260024767801859</v>
       </c>
       <c r="V25" s="19">
-        <f t="shared" ref="V25:V27" si="49">ABS(R25)/ABS(O25)</f>
+        <f t="shared" ref="V25:V27" si="50">ABS(R25)/ABS(O25)</f>
         <v>0.14296</v>
       </c>
       <c r="W25" s="19">
-        <f t="shared" ref="W25:W27" si="50">Q25/N25</f>
+        <f t="shared" ref="W25:W27" si="51">Q25/N25</f>
         <v>0.11761000000000001</v>
       </c>
       <c r="X25" s="20">
@@ -4030,7 +4030,7 @@
         <v>3.43</v>
       </c>
       <c r="AE25" s="20">
-        <f t="shared" ref="AE25:AE27" si="51">AD25+AC25+AB25</f>
+        <f t="shared" ref="AE25:AE27" si="52">AD25+AC25+AB25</f>
         <v>25.380000000000003</v>
       </c>
       <c r="AF25" s="45">
@@ -4043,7 +4043,7 @@
         <v>0</v>
       </c>
       <c r="AI25" s="45">
-        <f t="shared" ref="AI25:AI27" si="52">AF25+AG25+AH25</f>
+        <f t="shared" ref="AI25:AI27" si="53">AF25+AG25+AH25</f>
         <v>21.36</v>
       </c>
       <c r="AJ25" s="46">
@@ -4082,19 +4082,19 @@
         <v>157</v>
       </c>
       <c r="AU25" s="43">
-        <f t="shared" ref="AU25:AU27" si="53">AT25+AS25</f>
+        <f t="shared" ref="AU25:AU27" si="54">AT25+AS25</f>
         <v>22</v>
       </c>
       <c r="AV25" s="45">
-        <f t="shared" ref="AV25:AV27" si="54">AS25*0.11761</f>
+        <f t="shared" ref="AV25:AV27" si="55">AS25*0.11761</f>
         <v>-15.877350000000002</v>
       </c>
       <c r="AW25" s="45">
-        <f t="shared" ref="AW25:AW27" si="55">AT25*0.14296</f>
+        <f t="shared" ref="AW25:AW27" si="56">AT25*0.14296</f>
         <v>22.44472</v>
       </c>
       <c r="AX25" s="45">
-        <f t="shared" ref="AX25:AX27" si="56">AW25+AV25</f>
+        <f t="shared" ref="AX25:AX27" si="57">AW25+AV25</f>
         <v>6.5673699999999986</v>
       </c>
       <c r="AY25" s="45">
@@ -4105,7 +4105,7 @@
         <v>0.01</v>
       </c>
       <c r="BA25" s="20">
-        <f t="shared" ref="BA25:BA27" si="57">AZ25+AY25+AX25</f>
+        <f t="shared" ref="BA25:BA27" si="58">AZ25+AY25+AX25</f>
         <v>5.2273699999999987</v>
       </c>
       <c r="BB25" s="21">
@@ -4121,7 +4121,7 @@
         <v>0</v>
       </c>
       <c r="BF25" s="22">
-        <f t="shared" ref="BF25:BF27" si="58">BD25+BC25+BE25</f>
+        <f t="shared" ref="BF25:BF27" si="59">BD25+BC25+BE25</f>
         <v>11.36</v>
       </c>
     </row>
@@ -4138,7 +4138,7 @@
         <v>-605</v>
       </c>
       <c r="E26" s="15">
-        <f t="shared" ref="E26:E27" si="59">ROUND(K26/M26,0)</f>
+        <f t="shared" ref="E26:E27" si="60">ROUND(K26/M26,0)</f>
         <v>0</v>
       </c>
       <c r="F26" s="15">
@@ -4163,7 +4163,7 @@
         <v>-206</v>
       </c>
       <c r="M26" s="16">
-        <f t="shared" ref="M26" si="60">L26/F26</f>
+        <f t="shared" ref="M26" si="61">L26/F26</f>
         <v>0.34049586776859503</v>
       </c>
       <c r="N26" s="15">
@@ -4173,34 +4173,34 @@
         <v>214</v>
       </c>
       <c r="P26" s="15">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>358</v>
       </c>
       <c r="Q26" s="17">
-        <f t="shared" si="45"/>
+        <f t="shared" si="46"/>
         <v>16.935840000000002</v>
       </c>
       <c r="R26" s="17">
-        <f t="shared" si="46"/>
+        <f t="shared" si="47"/>
         <v>30.593440000000001</v>
       </c>
       <c r="S26" s="17">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>47.52928</v>
       </c>
       <c r="T26" s="17">
         <v>0</v>
       </c>
       <c r="U26" s="18">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v>0.13276335195530725</v>
       </c>
       <c r="V26" s="19">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>0.14296</v>
       </c>
       <c r="W26" s="19">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>0.11761000000000002</v>
       </c>
       <c r="X26" s="20">
@@ -4226,7 +4226,7 @@
         <v>8.11</v>
       </c>
       <c r="AE26" s="20">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>92.03</v>
       </c>
       <c r="AF26" s="17">
@@ -4239,7 +4239,7 @@
         <v>0</v>
       </c>
       <c r="AI26" s="17">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>22.14</v>
       </c>
       <c r="AJ26" s="47">
@@ -4250,11 +4250,11 @@
         <v>22.14</v>
       </c>
       <c r="AL26" s="15">
-        <f t="shared" ref="AL26:AM26" si="61">AS26-AO26</f>
+        <f t="shared" ref="AL26:AM26" si="62">AS26-AO26</f>
         <v>599</v>
       </c>
       <c r="AM26" s="15">
-        <f t="shared" si="61"/>
+        <f t="shared" si="62"/>
         <v>242</v>
       </c>
       <c r="AN26" s="15">
@@ -4282,19 +4282,19 @@
         <v>242</v>
       </c>
       <c r="AU26" s="15">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>442</v>
       </c>
       <c r="AV26" s="17">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>23.522000000000002</v>
       </c>
       <c r="AW26" s="17">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>34.596319999999999</v>
       </c>
       <c r="AX26" s="17">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>58.118319999999997</v>
       </c>
       <c r="AY26" s="17">
@@ -4304,7 +4304,7 @@
         <v>0.13</v>
       </c>
       <c r="BA26" s="20">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>58.24832</v>
       </c>
       <c r="BB26" s="21">
@@ -4320,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="BF26" s="22">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>12.14</v>
       </c>
     </row>
@@ -4333,33 +4333,33 @@
         <v>45673</v>
       </c>
       <c r="D27" s="15">
-        <f t="shared" ref="D27" si="62">ROUND(J27/M27,0)</f>
+        <f t="shared" ref="D27" si="63">ROUND(J27/M27,0)</f>
         <v>-309</v>
       </c>
       <c r="E27" s="15">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>0</v>
       </c>
       <c r="F27" s="15">
         <v>-309</v>
       </c>
       <c r="G27" s="15">
-        <f t="shared" ref="G27:H27" si="63">G28+G29</f>
+        <f t="shared" ref="G27:H27" si="64">G28+G29</f>
         <v>489</v>
       </c>
       <c r="H27" s="15">
-        <f t="shared" si="63"/>
+        <f t="shared" si="64"/>
         <v>332</v>
       </c>
       <c r="I27" s="15">
         <v>821</v>
       </c>
       <c r="J27" s="15">
-        <f t="shared" ref="J27:K27" si="64">J28+J29</f>
+        <f t="shared" ref="J27:K27" si="65">J28+J29</f>
         <v>-210</v>
       </c>
       <c r="K27" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="L27" s="15">
@@ -4376,34 +4376,34 @@
         <v>332</v>
       </c>
       <c r="P27" s="15">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v>611</v>
       </c>
       <c r="Q27" s="17">
-        <f t="shared" si="45"/>
+        <f t="shared" si="46"/>
         <v>32.813189999999999</v>
       </c>
       <c r="R27" s="17">
-        <f t="shared" si="46"/>
+        <f t="shared" si="47"/>
         <v>47.462720000000004</v>
       </c>
       <c r="S27" s="17">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>80.27591000000001</v>
       </c>
       <c r="T27" s="17">
         <v>0</v>
       </c>
       <c r="U27" s="18">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v>0.1313844680851064</v>
       </c>
       <c r="V27" s="19">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>0.14296</v>
       </c>
       <c r="W27" s="19">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>0.11760999999999999</v>
       </c>
       <c r="X27" s="20">
@@ -4429,7 +4429,7 @@
         <v>12.56</v>
       </c>
       <c r="AE27" s="20">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>172.51999999999998</v>
       </c>
       <c r="AF27" s="17">
@@ -4442,7 +4442,7 @@
         <v>0</v>
       </c>
       <c r="AI27" s="17">
-        <f t="shared" si="52"/>
+        <f t="shared" si="53"/>
         <v>22.53</v>
       </c>
       <c r="AJ27" s="47">
@@ -4453,11 +4453,11 @@
         <v>22.53</v>
       </c>
       <c r="AL27" s="15">
-        <f t="shared" ref="AL27:AM27" si="65">AS27-AO27</f>
+        <f t="shared" ref="AL27:AM27" si="66">AS27-AO27</f>
         <v>693</v>
       </c>
       <c r="AM27" s="15">
-        <f t="shared" si="65"/>
+        <f t="shared" si="66"/>
         <v>231</v>
       </c>
       <c r="AN27" s="15">
@@ -4485,19 +4485,19 @@
         <v>231</v>
       </c>
       <c r="AU27" s="15">
-        <f t="shared" si="53"/>
+        <f t="shared" si="54"/>
         <v>825</v>
       </c>
       <c r="AV27" s="17">
-        <f t="shared" si="54"/>
+        <f t="shared" si="55"/>
         <v>69.860340000000008</v>
       </c>
       <c r="AW27" s="17">
-        <f t="shared" si="55"/>
+        <f t="shared" si="56"/>
         <v>33.023760000000003</v>
       </c>
       <c r="AX27" s="17">
-        <f t="shared" si="56"/>
+        <f t="shared" si="57"/>
         <v>102.88410000000002</v>
       </c>
       <c r="AY27" s="17">
@@ -4507,7 +4507,7 @@
         <v>0.25</v>
       </c>
       <c r="BA27" s="20">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>103.13410000000002</v>
       </c>
       <c r="BB27" s="21">
@@ -4523,7 +4523,7 @@
         <v>0</v>
       </c>
       <c r="BF27" s="22">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>12.53</v>
       </c>
     </row>
@@ -4741,15 +4741,15 @@
         <v>-10</v>
       </c>
       <c r="U30" s="18">
-        <f t="shared" ref="U30:U31" si="66">(ABS(Q30)+ABS(R30))/(ABS(N30)+ABS(O30))</f>
+        <f t="shared" ref="U30:U31" si="67">(ABS(Q30)+ABS(R30))/(ABS(N30)+ABS(O30))</f>
         <v>0.12236459709379127</v>
       </c>
       <c r="V30" s="19">
-        <f t="shared" ref="V30:V31" si="67">ABS(R30)/ABS(O30)</f>
+        <f t="shared" ref="V30:V31" si="68">ABS(R30)/ABS(O30)</f>
         <v>0.14295774647887324</v>
       </c>
       <c r="W30" s="19">
-        <f t="shared" ref="W30:W31" si="68">Q30/N30</f>
+        <f t="shared" ref="W30:W31" si="69">Q30/N30</f>
         <v>0.11760975609756097</v>
       </c>
       <c r="X30" s="20">
@@ -4789,7 +4789,7 @@
         <v>0</v>
       </c>
       <c r="AI30" s="17">
-        <f t="shared" ref="AI30:AI31" si="69">AF30+AG30+AH30</f>
+        <f t="shared" ref="AI30:AI31" si="70">AF30+AG30+AH30</f>
         <v>21.36</v>
       </c>
       <c r="AJ30" s="47">
@@ -4800,22 +4800,22 @@
         <v>89.57</v>
       </c>
       <c r="AL30" s="15">
-        <f t="shared" ref="AL30:AM30" si="70">AS30-AO30</f>
+        <f t="shared" ref="AL30:AM30" si="71">AS30-AO30</f>
         <v>732</v>
       </c>
       <c r="AM30" s="15">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>9</v>
       </c>
       <c r="AN30" s="15">
         <v>741</v>
       </c>
       <c r="AO30" s="15">
-        <f>D30-J30</f>
+        <f t="shared" ref="AO30:AP33" si="72">D30-J30</f>
         <v>0</v>
       </c>
       <c r="AP30" s="15">
-        <f>E30-K30</f>
+        <f t="shared" si="72"/>
         <v>190</v>
       </c>
       <c r="AQ30" s="15">
@@ -4831,7 +4831,7 @@
         <v>199</v>
       </c>
       <c r="AU30" s="15">
-        <f t="shared" ref="AU30:AU32" si="71">AT30+AS30</f>
+        <f t="shared" ref="AU30:AU32" si="73">AT30+AS30</f>
         <v>931</v>
       </c>
       <c r="AV30" s="17">
@@ -4843,7 +4843,7 @@
         <v>28.44904</v>
       </c>
       <c r="AX30" s="17">
-        <f t="shared" ref="AX30:AX31" si="72">AW30+AV30</f>
+        <f t="shared" ref="AX30:AX31" si="74">AW30+AV30</f>
         <v>114.53955999999999</v>
       </c>
       <c r="AY30" s="17">
@@ -4853,7 +4853,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="BA30" s="20">
-        <f t="shared" ref="BA30:BA31" si="73">AZ30+AY30+AX30</f>
+        <f t="shared" ref="BA30:BA31" si="75">AZ30+AY30+AX30</f>
         <v>114.81956</v>
       </c>
       <c r="BB30" s="21">
@@ -4869,7 +4869,7 @@
         <v>0</v>
       </c>
       <c r="BF30" s="22">
-        <f t="shared" ref="BF30:BF31" si="74">BD30+BC30+BE30</f>
+        <f t="shared" ref="BF30:BF31" si="76">BD30+BC30+BE30</f>
         <v>88.07</v>
       </c>
     </row>
@@ -4893,22 +4893,22 @@
         <v>-762</v>
       </c>
       <c r="G31" s="15">
-        <f t="shared" ref="G31:H31" si="75">G32+G33</f>
+        <f t="shared" ref="G31:H31" si="77">G32+G33</f>
         <v>321</v>
       </c>
       <c r="H31" s="15">
-        <f t="shared" si="75"/>
+        <f t="shared" si="77"/>
         <v>286</v>
       </c>
       <c r="I31" s="15">
         <v>607</v>
       </c>
       <c r="J31" s="15">
-        <f t="shared" ref="J31:K31" si="76">J32+J33</f>
+        <f t="shared" ref="J31:K31" si="78">J32+J33</f>
         <v>-304</v>
       </c>
       <c r="K31" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="78"/>
         <v>-1</v>
       </c>
       <c r="L31" s="15">
@@ -4928,30 +4928,30 @@
         <v>302</v>
       </c>
       <c r="Q31" s="17">
-        <f t="shared" ref="Q31:S31" si="77">Q32+Q33</f>
+        <f t="shared" ref="Q31:S31" si="79">Q32+Q33</f>
         <v>1.9100000000000001</v>
       </c>
       <c r="R31" s="17">
-        <f t="shared" si="77"/>
+        <f t="shared" si="79"/>
         <v>38.949999999999996</v>
       </c>
       <c r="S31" s="17">
-        <f t="shared" si="77"/>
+        <f t="shared" si="79"/>
         <v>40.859999999999992</v>
       </c>
       <c r="T31" s="17">
         <v>0</v>
       </c>
       <c r="U31" s="18">
-        <f t="shared" si="66"/>
+        <f t="shared" si="67"/>
         <v>0.1352980132450331</v>
       </c>
       <c r="V31" s="19">
-        <f t="shared" si="67"/>
+        <f t="shared" si="68"/>
         <v>0.13666666666666666</v>
       </c>
       <c r="W31" s="19">
-        <f t="shared" si="68"/>
+        <f t="shared" si="69"/>
         <v>0.1123529411764706</v>
       </c>
       <c r="X31" s="20">
@@ -4989,7 +4989,7 @@
         <v>0</v>
       </c>
       <c r="AI31" s="17">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>21.82</v>
       </c>
       <c r="AJ31" s="15">
@@ -5000,22 +5000,22 @@
         <v>62.77</v>
       </c>
       <c r="AL31" s="15">
-        <f t="shared" ref="AL31:AM31" si="78">AS31-AO31</f>
+        <f t="shared" ref="AL31:AM31" si="80">AS31-AO31</f>
         <v>592</v>
       </c>
       <c r="AM31" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="80"/>
         <v>242</v>
       </c>
       <c r="AN31" s="15">
         <v>834</v>
       </c>
       <c r="AO31" s="15">
-        <f>D31-J31</f>
+        <f t="shared" si="72"/>
         <v>-456</v>
       </c>
       <c r="AP31" s="15">
-        <f>E31-K31</f>
+        <f t="shared" si="72"/>
         <v>-1</v>
       </c>
       <c r="AQ31" s="15">
@@ -5026,27 +5026,27 @@
         <v>0.59973753280839892</v>
       </c>
       <c r="AS31" s="15">
-        <f t="shared" ref="AS31:AT31" si="79">AS32+AS33</f>
+        <f t="shared" ref="AS31:AT31" si="81">AS32+AS33</f>
         <v>136</v>
       </c>
       <c r="AT31" s="15">
-        <f t="shared" si="79"/>
+        <f t="shared" si="81"/>
         <v>241</v>
       </c>
       <c r="AU31" s="15">
-        <f t="shared" si="71"/>
+        <f t="shared" si="73"/>
         <v>377</v>
       </c>
       <c r="AV31" s="17">
-        <f t="shared" ref="AV31:AW31" si="80">AV32+AV33</f>
+        <f t="shared" ref="AV31:AW31" si="82">AV32+AV33</f>
         <v>15.293426873</v>
       </c>
       <c r="AW31" s="17">
-        <f t="shared" si="80"/>
+        <f t="shared" si="82"/>
         <v>32.941085250999997</v>
       </c>
       <c r="AX31" s="17">
-        <f t="shared" si="72"/>
+        <f t="shared" si="74"/>
         <v>48.234512123999998</v>
       </c>
       <c r="AY31" s="17">
@@ -5056,7 +5056,7 @@
         <v>0.11</v>
       </c>
       <c r="BA31" s="20">
-        <f t="shared" si="73"/>
+        <f t="shared" si="75"/>
         <v>48.344512123999998</v>
       </c>
       <c r="BB31" s="21">
@@ -5073,7 +5073,7 @@
         <v>0</v>
       </c>
       <c r="BF31" s="22">
-        <f t="shared" si="74"/>
+        <f t="shared" si="76"/>
         <v>60.164512123999998</v>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
         <v>32.159999999999997</v>
       </c>
       <c r="S32" s="39">
-        <f t="shared" ref="S32:S33" si="81">Q32+R32</f>
+        <f t="shared" ref="S32:S33" si="83">Q32+R32</f>
         <v>33.739999999999995</v>
       </c>
       <c r="T32" s="36"/>
@@ -5152,11 +5152,11 @@
       </c>
       <c r="AN32" s="36"/>
       <c r="AO32" s="36">
-        <f>D32-J32</f>
+        <f t="shared" si="72"/>
         <v>-358</v>
       </c>
       <c r="AP32" s="36">
-        <f>E32-K32</f>
+        <f t="shared" si="72"/>
         <v>-1</v>
       </c>
       <c r="AQ32" s="38"/>
@@ -5168,7 +5168,7 @@
         <v>200.83330000000001</v>
       </c>
       <c r="AU32" s="36">
-        <f t="shared" si="71"/>
+        <f t="shared" si="73"/>
         <v>314.16660000000002</v>
       </c>
       <c r="AV32" s="39">
@@ -5233,7 +5233,7 @@
         <v>6.79</v>
       </c>
       <c r="S33" s="39">
-        <f t="shared" si="81"/>
+        <f t="shared" si="83"/>
         <v>7.12</v>
       </c>
       <c r="T33" s="36"/>
@@ -5264,11 +5264,11 @@
       </c>
       <c r="AN33" s="36"/>
       <c r="AO33" s="36">
-        <f>D33-J33</f>
+        <f t="shared" si="72"/>
         <v>-97</v>
       </c>
       <c r="AP33" s="36">
-        <f>E33-K33</f>
+        <f t="shared" si="72"/>
         <v>0</v>
       </c>
       <c r="AQ33" s="38"/>
@@ -5424,22 +5424,22 @@
         <v>207.22</v>
       </c>
       <c r="AL34" s="15">
-        <f t="shared" ref="AL34:AM34" si="82">AS34-AO34</f>
+        <f t="shared" ref="AL34:AM34" si="84">AS34-AO34</f>
         <v>582</v>
       </c>
       <c r="AM34" s="15">
-        <f t="shared" si="82"/>
+        <f t="shared" si="84"/>
         <v>212</v>
       </c>
       <c r="AN34" s="15">
         <v>794</v>
       </c>
       <c r="AO34" s="15">
-        <f t="shared" ref="AO34:AP34" si="83">D34-J34</f>
+        <f t="shared" ref="AO34:AP34" si="85">D34-J34</f>
         <v>-670</v>
       </c>
       <c r="AP34" s="15">
-        <f t="shared" si="83"/>
+        <f t="shared" si="85"/>
         <v>-60</v>
       </c>
       <c r="AQ34" s="15">

</xml_diff>

<commit_message>
moved some subcomponent values from september to where they should be given the totals in october
</commit_message>
<xml_diff>
--- a/python-notebooks/billing.xlsx
+++ b/python-notebooks/billing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/klowe/repos-personal/energy-project/python-notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{313C4873-0570-0147-BAB6-D67ED3061733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA7D4984-72A6-5C4E-9381-3DFB04C112F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="23960" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Billing" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="101">
   <si>
     <t>303A ADU</t>
   </si>
@@ -428,7 +428,7 @@
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -486,8 +486,15 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="26">
+  <fills count="25">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -622,12 +629,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor rgb="FFC1E4F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="2" tint="-4.9989318521683403E-2"/>
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
@@ -744,12 +745,9 @@
     <xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="6" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="6" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -769,6 +767,9 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -984,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BF1012"/>
+  <dimension ref="A1:BF1010"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
@@ -995,7 +996,7 @@
     <col min="13" max="13" width="11.6640625" customWidth="1"/>
     <col min="14" max="14" width="10.83203125" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
-    <col min="16" max="16" width="7.1640625" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" customWidth="1"/>
     <col min="17" max="17" width="10.83203125" customWidth="1"/>
     <col min="18" max="19" width="10.5" customWidth="1"/>
     <col min="20" max="25" width="10" customWidth="1"/>
@@ -1032,152 +1033,152 @@
       <c r="A2" t="s">
         <v>88</v>
       </c>
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71" t="s">
+      <c r="C2" s="67"/>
+      <c r="D2" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="71"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="71"/>
-      <c r="V2" s="71"/>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="71"/>
-      <c r="Z2" s="71"/>
-      <c r="AA2" s="71"/>
-      <c r="AB2" s="71"/>
-      <c r="AC2" s="71"/>
-      <c r="AD2" s="71"/>
-      <c r="AE2" s="71"/>
-      <c r="AF2" s="71"/>
-      <c r="AG2" s="71"/>
-      <c r="AH2" s="71"/>
-      <c r="AI2" s="71"/>
-      <c r="AJ2" s="71"/>
-      <c r="AK2" s="71"/>
-      <c r="AL2" s="72" t="s">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="72"/>
-      <c r="AN2" s="72"/>
-      <c r="AO2" s="72"/>
-      <c r="AP2" s="72"/>
-      <c r="AQ2" s="72"/>
-      <c r="AR2" s="72"/>
-      <c r="AS2" s="72"/>
-      <c r="AT2" s="72"/>
-      <c r="AU2" s="72"/>
-      <c r="AV2" s="72"/>
-      <c r="AW2" s="72"/>
-      <c r="AX2" s="72"/>
-      <c r="AY2" s="72"/>
-      <c r="AZ2" s="72"/>
-      <c r="BA2" s="72"/>
-      <c r="BB2" s="72"/>
-      <c r="BC2" s="72"/>
-      <c r="BD2" s="72"/>
-      <c r="BE2" s="72"/>
-      <c r="BF2" s="72"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="68"/>
+      <c r="H2" s="68"/>
+      <c r="I2" s="68"/>
+      <c r="J2" s="68"/>
+      <c r="K2" s="68"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="68"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="68"/>
+      <c r="P2" s="68"/>
+      <c r="Q2" s="68"/>
+      <c r="R2" s="68"/>
+      <c r="S2" s="68"/>
+      <c r="T2" s="68"/>
+      <c r="U2" s="68"/>
+      <c r="V2" s="68"/>
+      <c r="W2" s="68"/>
+      <c r="X2" s="68"/>
+      <c r="Y2" s="68"/>
+      <c r="Z2" s="68"/>
+      <c r="AA2" s="68"/>
+      <c r="AB2" s="68"/>
+      <c r="AC2" s="68"/>
+      <c r="AD2" s="68"/>
+      <c r="AE2" s="68"/>
+      <c r="AF2" s="68"/>
+      <c r="AG2" s="68"/>
+      <c r="AH2" s="68"/>
+      <c r="AI2" s="68"/>
+      <c r="AJ2" s="68"/>
+      <c r="AK2" s="68"/>
+      <c r="AL2" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="69"/>
+      <c r="AN2" s="69"/>
+      <c r="AO2" s="69"/>
+      <c r="AP2" s="69"/>
+      <c r="AQ2" s="69"/>
+      <c r="AR2" s="69"/>
+      <c r="AS2" s="69"/>
+      <c r="AT2" s="69"/>
+      <c r="AU2" s="69"/>
+      <c r="AV2" s="69"/>
+      <c r="AW2" s="69"/>
+      <c r="AX2" s="69"/>
+      <c r="AY2" s="69"/>
+      <c r="AZ2" s="69"/>
+      <c r="BA2" s="69"/>
+      <c r="BB2" s="69"/>
+      <c r="BC2" s="69"/>
+      <c r="BD2" s="69"/>
+      <c r="BE2" s="69"/>
+      <c r="BF2" s="69"/>
     </row>
     <row r="3" spans="1:58" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="70" t="s">
+      <c r="B3" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="76" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="73" t="s">
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="74"/>
-      <c r="I3" s="74"/>
-      <c r="J3" s="73" t="s">
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="70" t="s">
         <v>91</v>
       </c>
-      <c r="K3" s="74"/>
-      <c r="L3" s="74"/>
-      <c r="M3" s="74"/>
-      <c r="N3" s="73" t="s">
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="74"/>
-      <c r="P3" s="74"/>
-      <c r="Q3" s="75" t="s">
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
+      <c r="Q3" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="R3" s="74"/>
-      <c r="S3" s="74"/>
-      <c r="T3" s="74"/>
-      <c r="U3" s="74"/>
-      <c r="V3" s="74"/>
-      <c r="W3" s="74"/>
-      <c r="X3" s="74"/>
-      <c r="Y3" s="74"/>
-      <c r="Z3" s="74"/>
-      <c r="AA3" s="74"/>
-      <c r="AB3" s="73" t="s">
+      <c r="R3" s="71"/>
+      <c r="S3" s="71"/>
+      <c r="T3" s="71"/>
+      <c r="U3" s="71"/>
+      <c r="V3" s="71"/>
+      <c r="W3" s="71"/>
+      <c r="X3" s="71"/>
+      <c r="Y3" s="71"/>
+      <c r="Z3" s="71"/>
+      <c r="AA3" s="71"/>
+      <c r="AB3" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="AC3" s="74"/>
-      <c r="AD3" s="74"/>
-      <c r="AE3" s="74"/>
-      <c r="AF3" s="74"/>
-      <c r="AG3" s="74"/>
-      <c r="AH3" s="74"/>
-      <c r="AI3" s="74"/>
+      <c r="AC3" s="71"/>
+      <c r="AD3" s="71"/>
+      <c r="AE3" s="71"/>
+      <c r="AF3" s="71"/>
+      <c r="AG3" s="71"/>
+      <c r="AH3" s="71"/>
+      <c r="AI3" s="71"/>
       <c r="AJ3" s="54" t="s">
         <v>6</v>
       </c>
       <c r="AK3" s="55"/>
-      <c r="AL3" s="73" t="s">
+      <c r="AL3" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="AM3" s="74"/>
-      <c r="AN3" s="74"/>
-      <c r="AO3" s="73" t="s">
+      <c r="AM3" s="71"/>
+      <c r="AN3" s="71"/>
+      <c r="AO3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="AP3" s="74"/>
-      <c r="AQ3" s="74"/>
-      <c r="AR3" s="74"/>
-      <c r="AS3" s="73" t="s">
+      <c r="AP3" s="71"/>
+      <c r="AQ3" s="71"/>
+      <c r="AR3" s="71"/>
+      <c r="AS3" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="AT3" s="74"/>
-      <c r="AU3" s="74"/>
-      <c r="AV3" s="75" t="s">
+      <c r="AT3" s="71"/>
+      <c r="AU3" s="71"/>
+      <c r="AV3" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="AW3" s="74"/>
-      <c r="AX3" s="74"/>
-      <c r="AY3" s="74"/>
-      <c r="AZ3" s="74"/>
-      <c r="BA3" s="74"/>
-      <c r="BB3" s="74"/>
-      <c r="BC3" s="74"/>
+      <c r="AW3" s="71"/>
+      <c r="AX3" s="71"/>
+      <c r="AY3" s="71"/>
+      <c r="AZ3" s="71"/>
+      <c r="BA3" s="71"/>
+      <c r="BB3" s="71"/>
+      <c r="BC3" s="71"/>
       <c r="BD3" s="54" t="s">
         <v>8</v>
       </c>
@@ -2916,7 +2917,7 @@
       <c r="AN15" s="62"/>
       <c r="AO15" s="63"/>
       <c r="AP15" s="62"/>
-      <c r="AQ15" s="66"/>
+      <c r="AQ15" s="65"/>
       <c r="AR15" s="38"/>
       <c r="AS15" s="36">
         <v>-64.965500000000006</v>
@@ -2977,7 +2978,7 @@
         <v>-28.712348573999996</v>
       </c>
       <c r="R16" s="39">
-        <f t="shared" ref="R16:R17" si="31">O16*0.20001</f>
+        <f t="shared" ref="R16" si="31">O16*0.20001</f>
         <v>3.5587979309999995</v>
       </c>
       <c r="S16" s="39"/>
@@ -3004,7 +3005,7 @@
       <c r="AN16" s="62"/>
       <c r="AO16" s="63"/>
       <c r="AP16" s="62"/>
-      <c r="AQ16" s="66"/>
+      <c r="AQ16" s="65"/>
       <c r="AR16" s="38"/>
       <c r="AS16" s="36">
         <v>-249.03450000000001</v>
@@ -3079,13 +3080,13 @@
         <f>L17/F17</f>
         <v>0.28825857519788917</v>
       </c>
-      <c r="N17" s="67">
+      <c r="N17" s="76">
         <v>-211</v>
       </c>
-      <c r="O17" s="67">
+      <c r="O17" s="76">
         <v>95</v>
       </c>
-      <c r="P17" s="67">
+      <c r="P17" s="76">
         <f>O17+N17</f>
         <v>-116</v>
       </c>
@@ -3094,7 +3095,7 @@
         <v>-25.56476</v>
       </c>
       <c r="R17" s="17">
-        <f t="shared" si="31"/>
+        <f>O17*0.20001</f>
         <v>19.00095</v>
       </c>
       <c r="S17" s="17">
@@ -3269,9 +3270,9 @@
       </c>
       <c r="L18" s="36"/>
       <c r="M18" s="38"/>
-      <c r="N18" s="68"/>
-      <c r="O18" s="68"/>
-      <c r="P18" s="68"/>
+      <c r="N18" s="66"/>
+      <c r="O18" s="66"/>
+      <c r="P18" s="66"/>
       <c r="Q18" s="39"/>
       <c r="R18" s="39"/>
       <c r="S18" s="39"/>
@@ -3345,9 +3346,9 @@
       </c>
       <c r="L19" s="36"/>
       <c r="M19" s="38"/>
-      <c r="N19" s="68"/>
-      <c r="O19" s="68"/>
-      <c r="P19" s="68"/>
+      <c r="N19" s="66"/>
+      <c r="O19" s="66"/>
+      <c r="P19" s="66"/>
       <c r="Q19" s="39"/>
       <c r="R19" s="39"/>
       <c r="S19" s="39"/>
@@ -3379,8 +3380,8 @@
       <c r="AS19" s="36"/>
       <c r="AT19" s="36"/>
       <c r="AU19" s="36"/>
-      <c r="AV19" s="39"/>
-      <c r="AW19" s="39"/>
+      <c r="AV19" s="36"/>
+      <c r="AW19" s="36"/>
       <c r="AX19" s="39"/>
       <c r="AY19" s="39"/>
       <c r="AZ19" s="39"/>
@@ -3392,126 +3393,261 @@
       <c r="BF19" s="39"/>
     </row>
     <row r="20" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="69">
-        <v>-145</v>
-      </c>
-      <c r="O20" s="69">
-        <v>69</v>
-      </c>
-      <c r="P20" s="69">
-        <f t="shared" ref="P20:P22" si="36">O20+N20</f>
-        <v>-76</v>
-      </c>
-      <c r="Q20" s="27">
-        <f>N20*0.12116</f>
-        <v>-17.568200000000001</v>
-      </c>
-      <c r="R20" s="27">
-        <f>O20*0.20001</f>
-        <v>13.800689999999999</v>
-      </c>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
-      <c r="V20" s="27"/>
-      <c r="W20" s="27"/>
-      <c r="X20" s="27"/>
-      <c r="Y20" s="27"/>
-      <c r="Z20" s="27"/>
-      <c r="AA20" s="27"/>
-      <c r="AB20" s="27"/>
-      <c r="AC20" s="27"/>
-      <c r="AD20" s="27"/>
-      <c r="AE20" s="27"/>
-      <c r="AF20" s="27"/>
-      <c r="AG20" s="27"/>
-      <c r="AH20" s="27"/>
-      <c r="AI20" s="27"/>
-      <c r="AJ20" s="27"/>
-      <c r="AK20" s="56"/>
-      <c r="AL20" s="57"/>
-      <c r="AM20" s="57"/>
-      <c r="AN20" s="58"/>
-      <c r="AO20" s="57"/>
-      <c r="AP20" s="58"/>
-      <c r="AQ20" s="66"/>
-      <c r="AR20" s="26"/>
-      <c r="AS20" s="25">
-        <v>-275</v>
-      </c>
-      <c r="AT20" s="25">
-        <v>99</v>
-      </c>
-      <c r="AU20" s="25">
-        <f t="shared" ref="AU20:AU22" si="37">AT20+AS20</f>
-        <v>-176</v>
-      </c>
-      <c r="AV20" s="27">
-        <f>AS20*0.12116</f>
-        <v>-33.319000000000003</v>
-      </c>
-      <c r="AW20" s="27">
-        <f>AT20*0.20001</f>
-        <v>19.800989999999999</v>
-      </c>
-      <c r="AX20" s="56"/>
-      <c r="AY20" s="56"/>
-      <c r="AZ20" s="56"/>
-      <c r="BA20" s="64"/>
-      <c r="BB20" s="64"/>
-      <c r="BC20" s="64"/>
-      <c r="BD20" s="64"/>
-      <c r="BE20" s="56"/>
-      <c r="BF20" s="56"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="13">
+        <v>45571</v>
+      </c>
+      <c r="C20" s="13">
+        <v>45581</v>
+      </c>
+      <c r="D20" s="15">
+        <f>ROUND(J20/M20,0)</f>
+        <v>-1199</v>
+      </c>
+      <c r="E20" s="15">
+        <f>ROUND(K20/M20,0)</f>
+        <v>-93</v>
+      </c>
+      <c r="F20" s="15">
+        <v>-1292</v>
+      </c>
+      <c r="G20" s="15">
+        <f t="shared" ref="G20:H20" si="36">G21+G22</f>
+        <v>191</v>
+      </c>
+      <c r="H20" s="15">
+        <f t="shared" si="36"/>
+        <v>157</v>
+      </c>
+      <c r="I20" s="15">
+        <v>348</v>
+      </c>
+      <c r="J20" s="15">
+        <f t="shared" ref="J20:K20" si="37">J21+J22</f>
+        <v>-334</v>
+      </c>
+      <c r="K20" s="15">
+        <f t="shared" si="37"/>
+        <v>-26</v>
+      </c>
+      <c r="L20" s="15">
+        <v>-360</v>
+      </c>
+      <c r="M20" s="16">
+        <f>L20/F20</f>
+        <v>0.27863777089783281</v>
+      </c>
+      <c r="N20" s="15">
+        <f>N22+N21</f>
+        <v>-143</v>
+      </c>
+      <c r="O20" s="15">
+        <f>O22+O21</f>
+        <v>131</v>
+      </c>
+      <c r="P20" s="15">
+        <f t="shared" ref="P20" si="38">O20+N20</f>
+        <v>-12</v>
+      </c>
+      <c r="Q20" s="17">
+        <f>Q21+Q22</f>
+        <v>-17.332979999999999</v>
+      </c>
+      <c r="R20" s="17">
+        <f>R21+R22</f>
+        <v>22.664209999999997</v>
+      </c>
+      <c r="S20" s="17">
+        <f>R20+Q20</f>
+        <v>5.3312299999999979</v>
+      </c>
+      <c r="T20" s="17">
+        <f>N21*0.01</f>
+        <v>-1.45</v>
+      </c>
+      <c r="U20" s="18">
+        <f>(ABS(Q20)+ABS(R20))/(ABS(N20)+ABS(O20))</f>
+        <v>0.14597514598540146</v>
+      </c>
+      <c r="V20" s="19">
+        <f>ABS(R20)/ABS(O20)</f>
+        <v>0.17300923664122136</v>
+      </c>
+      <c r="W20" s="19">
+        <f>Q20/N20</f>
+        <v>0.12120965034965034</v>
+      </c>
+      <c r="X20" s="20">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="20">
+        <f>Q20+R20+T20+X20</f>
+        <v>3.8812299999999977</v>
+      </c>
+      <c r="Z20" s="21">
+        <v>163.22999999999999</v>
+      </c>
+      <c r="AA20" s="21">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="17">
+        <v>4.42</v>
+      </c>
+      <c r="AC20" s="17">
+        <v>1.01</v>
+      </c>
+      <c r="AD20" s="17">
+        <v>2.1</v>
+      </c>
+      <c r="AE20" s="20">
+        <f>AD20+AC20+AB20</f>
+        <v>7.53</v>
+      </c>
+      <c r="AF20" s="17">
+        <v>10</v>
+      </c>
+      <c r="AG20" s="17">
+        <v>12.14</v>
+      </c>
+      <c r="AH20" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI20" s="17">
+        <f>AF20+AG20+AH20</f>
+        <v>22.14</v>
+      </c>
+      <c r="AJ20" s="17">
+        <v>-55.17</v>
+      </c>
+      <c r="AK20" s="22">
+        <f>AA20+AI20+AJ20</f>
+        <v>-33.03</v>
+      </c>
+      <c r="AL20" s="15">
+        <f t="shared" ref="AL20:AM20" si="39">AS20-AO20</f>
+        <v>544</v>
+      </c>
+      <c r="AM20" s="15">
+        <f t="shared" si="39"/>
+        <v>199</v>
+      </c>
+      <c r="AN20" s="15">
+        <v>743</v>
+      </c>
+      <c r="AO20" s="15">
+        <f>D20-J20</f>
+        <v>-865</v>
+      </c>
+      <c r="AP20" s="15">
+        <f>E20-K20</f>
+        <v>-67</v>
+      </c>
+      <c r="AQ20" s="15">
+        <v>-932</v>
+      </c>
+      <c r="AR20" s="16">
+        <f>AQ20/F20</f>
+        <v>0.72136222910216719</v>
+      </c>
+      <c r="AS20" s="15">
+        <f>AS21+AS22</f>
+        <v>-321</v>
+      </c>
+      <c r="AT20" s="15">
+        <f>AT22+AT21</f>
+        <v>132</v>
+      </c>
+      <c r="AU20" s="15">
+        <f t="shared" ref="AU20" si="40">AT20+AS20</f>
+        <v>-189</v>
+      </c>
+      <c r="AV20" s="17">
+        <f>AV21+AV22</f>
+        <v>-38.729060000000004</v>
+      </c>
+      <c r="AW20" s="17">
+        <f>AW21+AW22</f>
+        <v>24.51867</v>
+      </c>
+      <c r="AX20" s="17">
+        <f>AW20+AV20</f>
+        <v>-14.210390000000004</v>
+      </c>
+      <c r="AY20" s="17">
+        <f>(AS21+AS22)*0.01</f>
+        <v>-3.21</v>
+      </c>
+      <c r="AZ20" s="17">
+        <v>0</v>
+      </c>
+      <c r="BA20" s="20">
+        <f>AZ20+AY20+AX20</f>
+        <v>-17.420390000000005</v>
+      </c>
+      <c r="BB20" s="21">
+        <v>204.71</v>
+      </c>
+      <c r="BC20" s="21">
+        <v>0</v>
+      </c>
+      <c r="BD20" s="20">
+        <v>12.14</v>
+      </c>
+      <c r="BE20" s="17">
+        <v>-55.17</v>
+      </c>
+      <c r="BF20" s="22">
+        <f t="shared" ref="BF20" si="41">BD20+BC20+BE20</f>
+        <v>-43.03</v>
+      </c>
     </row>
     <row r="21" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="25">
+        <f>ROUND(J21/M20,0)</f>
+        <v>-983</v>
+      </c>
+      <c r="E21" s="25">
+        <f>ROUND(K21/M20,0)</f>
+        <v>-83</v>
+      </c>
       <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
+      <c r="G21" s="25">
+        <v>129</v>
+      </c>
+      <c r="H21" s="25">
+        <v>92</v>
+      </c>
       <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
+      <c r="J21" s="25">
+        <v>-274</v>
+      </c>
+      <c r="K21" s="25">
+        <v>-23</v>
+      </c>
       <c r="L21" s="25"/>
       <c r="M21" s="26"/>
-      <c r="N21" s="69">
-        <v>2</v>
-      </c>
-      <c r="O21" s="69">
-        <v>62</v>
-      </c>
-      <c r="P21" s="69">
-        <f t="shared" si="36"/>
-        <v>64</v>
+      <c r="N21" s="75">
+        <v>-145</v>
+      </c>
+      <c r="O21" s="75">
+        <v>69</v>
+      </c>
+      <c r="P21" s="75">
+        <f>O21+N21</f>
+        <v>-76</v>
       </c>
       <c r="Q21" s="27">
-        <f>N21*0.11761</f>
-        <v>0.23522000000000001</v>
+        <f>N21*0.12116</f>
+        <v>-17.568200000000001</v>
       </c>
       <c r="R21" s="27">
-        <f>O21*0.14296</f>
-        <v>8.8635199999999994</v>
+        <f>O21*0.20001</f>
+        <v>13.800689999999999</v>
       </c>
       <c r="S21" s="27"/>
       <c r="T21" s="27"/>
@@ -3530,2019 +3666,1763 @@
       <c r="AG21" s="27"/>
       <c r="AH21" s="27"/>
       <c r="AI21" s="27"/>
-      <c r="AJ21" s="27"/>
-      <c r="AK21" s="56"/>
-      <c r="AL21" s="57"/>
-      <c r="AM21" s="57"/>
-      <c r="AN21" s="58"/>
-      <c r="AO21" s="57"/>
-      <c r="AP21" s="58"/>
-      <c r="AQ21" s="66"/>
+      <c r="AJ21" s="41"/>
+      <c r="AK21" s="27"/>
+      <c r="AL21" s="25"/>
+      <c r="AM21" s="25"/>
+      <c r="AN21" s="25"/>
+      <c r="AO21" s="25"/>
+      <c r="AP21" s="25"/>
+      <c r="AQ21" s="25"/>
       <c r="AR21" s="26"/>
       <c r="AS21" s="25">
-        <v>-46</v>
+        <v>-275</v>
       </c>
       <c r="AT21" s="25">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="AU21" s="25">
-        <f t="shared" si="37"/>
-        <v>-13</v>
+        <f>AT21+AS21</f>
+        <v>-176</v>
       </c>
       <c r="AV21" s="27">
-        <f>AS21*0.11761</f>
-        <v>-5.4100600000000005</v>
+        <f>AS21*0.12116</f>
+        <v>-33.319000000000003</v>
       </c>
       <c r="AW21" s="27">
-        <f>AT21*0.14296</f>
-        <v>4.7176800000000005</v>
-      </c>
-      <c r="AX21" s="56"/>
-      <c r="AY21" s="56"/>
-      <c r="AZ21" s="56"/>
-      <c r="BA21" s="64"/>
-      <c r="BB21" s="64"/>
-      <c r="BC21" s="64"/>
-      <c r="BD21" s="64"/>
-      <c r="BE21" s="56"/>
-      <c r="BF21" s="56"/>
+        <f>AT21*0.20001</f>
+        <v>19.800989999999999</v>
+      </c>
+      <c r="AX21" s="27"/>
+      <c r="AY21" s="27"/>
+      <c r="AZ21" s="27"/>
+      <c r="BA21" s="27"/>
+      <c r="BB21" s="27"/>
+      <c r="BC21" s="27"/>
+      <c r="BD21" s="27"/>
+      <c r="BE21" s="27"/>
+      <c r="BF21" s="27"/>
     </row>
     <row r="22" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="2"/>
-      <c r="B22" s="13">
-        <v>45571</v>
-      </c>
-      <c r="C22" s="13">
-        <v>45581</v>
-      </c>
-      <c r="D22" s="15">
-        <f>ROUND(J22/M22,0)</f>
-        <v>-1199</v>
-      </c>
-      <c r="E22" s="15">
-        <f>ROUND(K22/M22,0)</f>
-        <v>-93</v>
-      </c>
-      <c r="F22" s="15">
-        <v>-1292</v>
-      </c>
-      <c r="G22" s="15">
-        <f t="shared" ref="G22:H22" si="38">G23+G24</f>
-        <v>191</v>
-      </c>
-      <c r="H22" s="15">
-        <f t="shared" si="38"/>
-        <v>157</v>
-      </c>
-      <c r="I22" s="15">
-        <v>348</v>
-      </c>
-      <c r="J22" s="15">
-        <f t="shared" ref="J22:K22" si="39">J23+J24</f>
-        <v>-334</v>
-      </c>
-      <c r="K22" s="15">
-        <f t="shared" si="39"/>
-        <v>-26</v>
-      </c>
-      <c r="L22" s="15">
-        <v>-360</v>
-      </c>
-      <c r="M22" s="16">
-        <f>L22/F22</f>
-        <v>0.27863777089783281</v>
-      </c>
-      <c r="N22" s="15">
-        <f t="shared" ref="N22:O22" si="40">N21+N20</f>
-        <v>-143</v>
-      </c>
-      <c r="O22" s="15">
-        <f t="shared" si="40"/>
-        <v>131</v>
-      </c>
-      <c r="P22" s="15">
-        <f t="shared" si="36"/>
-        <v>-12</v>
-      </c>
-      <c r="Q22" s="17">
-        <f t="shared" ref="Q22:R22" si="41">Q20+Q21</f>
-        <v>-17.332979999999999</v>
-      </c>
-      <c r="R22" s="17">
-        <f t="shared" si="41"/>
-        <v>22.664209999999997</v>
-      </c>
-      <c r="S22" s="17">
-        <f>R22+Q22</f>
-        <v>5.3312299999999979</v>
-      </c>
-      <c r="T22" s="17">
-        <f>N20*0.01</f>
-        <v>-1.45</v>
-      </c>
-      <c r="U22" s="18">
-        <f>(ABS(Q22)+ABS(R22))/(ABS(N22)+ABS(O22))</f>
-        <v>0.14597514598540146</v>
-      </c>
-      <c r="V22" s="19">
-        <f>ABS(R22)/ABS(O22)</f>
-        <v>0.17300923664122136</v>
-      </c>
-      <c r="W22" s="19">
-        <f>Q22/N22</f>
-        <v>0.12120965034965034</v>
-      </c>
-      <c r="X22" s="20">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="20">
-        <f>Q22+R22+T22+X22</f>
-        <v>3.8812299999999977</v>
-      </c>
-      <c r="Z22" s="21">
-        <v>163.22999999999999</v>
-      </c>
-      <c r="AA22" s="21">
-        <v>0</v>
-      </c>
-      <c r="AB22" s="17">
-        <v>4.42</v>
-      </c>
-      <c r="AC22" s="17">
-        <v>1.01</v>
-      </c>
-      <c r="AD22" s="17">
-        <v>2.1</v>
-      </c>
-      <c r="AE22" s="20">
-        <f>AD22+AC22+AB22</f>
-        <v>7.53</v>
-      </c>
-      <c r="AF22" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG22" s="17">
-        <v>12.14</v>
-      </c>
-      <c r="AH22" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI22" s="17">
-        <f>AF22+AG22+AH22</f>
-        <v>22.14</v>
-      </c>
-      <c r="AJ22" s="17">
-        <v>-55.17</v>
-      </c>
-      <c r="AK22" s="22">
-        <f>AA22+AI22+AJ22</f>
-        <v>-33.03</v>
-      </c>
-      <c r="AL22" s="15">
-        <f t="shared" ref="AL22:AM22" si="42">AS22-AO22</f>
-        <v>544</v>
-      </c>
-      <c r="AM22" s="15">
-        <f t="shared" si="42"/>
-        <v>199</v>
-      </c>
-      <c r="AN22" s="15">
-        <v>743</v>
-      </c>
-      <c r="AO22" s="15">
-        <f>D22-J22</f>
-        <v>-865</v>
-      </c>
-      <c r="AP22" s="15">
-        <f>E22-K22</f>
-        <v>-67</v>
-      </c>
-      <c r="AQ22" s="15">
-        <v>-932</v>
-      </c>
-      <c r="AR22" s="16">
-        <f>AQ22/F22</f>
-        <v>0.72136222910216719</v>
-      </c>
-      <c r="AS22" s="15">
-        <f>AS20+AS21</f>
-        <v>-321</v>
-      </c>
-      <c r="AT22" s="15">
-        <f>AT21+AT20</f>
-        <v>132</v>
-      </c>
-      <c r="AU22" s="15">
-        <f t="shared" si="37"/>
-        <v>-189</v>
-      </c>
-      <c r="AV22" s="17">
-        <f t="shared" ref="AV22:AW22" si="43">AV20+AV21</f>
-        <v>-38.729060000000004</v>
-      </c>
-      <c r="AW22" s="17">
-        <f t="shared" si="43"/>
-        <v>24.51867</v>
-      </c>
-      <c r="AX22" s="17">
-        <f>AW22+AV22</f>
-        <v>-14.210390000000004</v>
-      </c>
-      <c r="AY22" s="17">
-        <f>(AS20+AS21)*0.01</f>
-        <v>-3.21</v>
-      </c>
-      <c r="AZ22" s="17">
-        <v>0</v>
-      </c>
-      <c r="BA22" s="20">
-        <f>AZ22+AY22+AX22</f>
-        <v>-17.420390000000005</v>
-      </c>
-      <c r="BB22" s="21">
-        <v>204.71</v>
-      </c>
-      <c r="BC22" s="21">
-        <v>0</v>
-      </c>
-      <c r="BD22" s="20">
-        <v>12.14</v>
-      </c>
-      <c r="BE22" s="17">
-        <v>-55.17</v>
-      </c>
-      <c r="BF22" s="22">
-        <f t="shared" ref="BF22" si="44">BD22+BC22+BE22</f>
-        <v>-43.03</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="25">
+        <f>ROUND(J22/M20,0)</f>
+        <v>-215</v>
+      </c>
+      <c r="E22" s="25">
+        <f>ROUND(K22/M20,0)</f>
+        <v>-11</v>
+      </c>
+      <c r="F22" s="25"/>
+      <c r="G22" s="25">
+        <v>62</v>
+      </c>
+      <c r="H22" s="25">
+        <v>65</v>
+      </c>
+      <c r="I22" s="25"/>
+      <c r="J22" s="25">
+        <v>-60</v>
+      </c>
+      <c r="K22" s="25">
+        <v>-3</v>
+      </c>
+      <c r="L22" s="25"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="75">
+        <v>2</v>
+      </c>
+      <c r="O22" s="75">
+        <v>62</v>
+      </c>
+      <c r="P22" s="75">
+        <f>O22+N22</f>
+        <v>64</v>
+      </c>
+      <c r="Q22" s="27">
+        <f>N22*0.11761</f>
+        <v>0.23522000000000001</v>
+      </c>
+      <c r="R22" s="27">
+        <f>O22*0.14296</f>
+        <v>8.8635199999999994</v>
+      </c>
+      <c r="S22" s="27"/>
+      <c r="T22" s="27"/>
+      <c r="U22" s="27"/>
+      <c r="V22" s="27"/>
+      <c r="W22" s="27"/>
+      <c r="X22" s="27"/>
+      <c r="Y22" s="27"/>
+      <c r="Z22" s="27"/>
+      <c r="AA22" s="27"/>
+      <c r="AB22" s="27"/>
+      <c r="AC22" s="27"/>
+      <c r="AD22" s="27"/>
+      <c r="AE22" s="27"/>
+      <c r="AF22" s="27"/>
+      <c r="AG22" s="27"/>
+      <c r="AH22" s="27"/>
+      <c r="AI22" s="27"/>
+      <c r="AJ22" s="41"/>
+      <c r="AK22" s="27"/>
+      <c r="AL22" s="25"/>
+      <c r="AM22" s="25"/>
+      <c r="AN22" s="25"/>
+      <c r="AO22" s="25"/>
+      <c r="AP22" s="25"/>
+      <c r="AQ22" s="25"/>
+      <c r="AR22" s="26"/>
+      <c r="AS22" s="25">
+        <v>-46</v>
+      </c>
+      <c r="AT22" s="25">
+        <v>33</v>
+      </c>
+      <c r="AU22" s="25">
+        <f>AT22+AS22</f>
+        <v>-13</v>
+      </c>
+      <c r="AV22" s="27">
+        <f>AS22*0.11761</f>
+        <v>-5.4100600000000005</v>
+      </c>
+      <c r="AW22" s="27">
+        <f>AT22*0.14296</f>
+        <v>4.7176800000000005</v>
+      </c>
+      <c r="AX22" s="27"/>
+      <c r="AY22" s="27"/>
+      <c r="AZ22" s="27"/>
+      <c r="BA22" s="27"/>
+      <c r="BB22" s="27"/>
+      <c r="BC22" s="27"/>
+      <c r="BD22" s="27"/>
+      <c r="BE22" s="27"/>
+      <c r="BF22" s="27"/>
     </row>
     <row r="23" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="40"/>
-      <c r="C23" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" s="25">
-        <f>ROUND(J23/M22,0)</f>
-        <v>-983</v>
-      </c>
-      <c r="E23" s="25">
-        <f>ROUND(K23/M22,0)</f>
-        <v>-83</v>
-      </c>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25">
-        <v>129</v>
-      </c>
-      <c r="H23" s="25">
-        <v>92</v>
-      </c>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25">
-        <v>-274</v>
-      </c>
-      <c r="K23" s="25">
-        <v>-23</v>
-      </c>
-      <c r="L23" s="25"/>
-      <c r="M23" s="26"/>
-      <c r="N23" s="25"/>
-      <c r="O23" s="25"/>
-      <c r="P23" s="25"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
-      <c r="V23" s="27"/>
-      <c r="W23" s="27"/>
-      <c r="X23" s="27"/>
-      <c r="Y23" s="27"/>
-      <c r="Z23" s="27"/>
-      <c r="AA23" s="27"/>
-      <c r="AB23" s="27"/>
-      <c r="AC23" s="27"/>
-      <c r="AD23" s="27"/>
-      <c r="AE23" s="27"/>
-      <c r="AF23" s="27"/>
-      <c r="AG23" s="27"/>
-      <c r="AH23" s="27"/>
-      <c r="AI23" s="27"/>
-      <c r="AJ23" s="41"/>
-      <c r="AK23" s="27"/>
-      <c r="AL23" s="25"/>
-      <c r="AM23" s="25"/>
-      <c r="AN23" s="25"/>
-      <c r="AO23" s="25"/>
-      <c r="AP23" s="25"/>
-      <c r="AQ23" s="25"/>
-      <c r="AR23" s="26"/>
-      <c r="AS23" s="25"/>
-      <c r="AT23" s="25"/>
-      <c r="AU23" s="25"/>
-      <c r="AV23" s="27"/>
-      <c r="AW23" s="27"/>
-      <c r="AX23" s="27"/>
-      <c r="AY23" s="27"/>
-      <c r="AZ23" s="27"/>
-      <c r="BA23" s="27"/>
-      <c r="BB23" s="27"/>
-      <c r="BC23" s="27"/>
-      <c r="BD23" s="27"/>
-      <c r="BE23" s="27"/>
-      <c r="BF23" s="27"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="42">
+        <v>45600</v>
+      </c>
+      <c r="C23" s="42">
+        <v>45610</v>
+      </c>
+      <c r="D23" s="43">
+        <f>ROUND(J23/M23,0)</f>
+        <v>-973</v>
+      </c>
+      <c r="E23" s="43">
+        <f>ROUND(K23/M23,0)</f>
+        <v>-17</v>
+      </c>
+      <c r="F23" s="43">
+        <v>-990</v>
+      </c>
+      <c r="G23" s="43">
+        <v>219</v>
+      </c>
+      <c r="H23" s="43">
+        <v>197</v>
+      </c>
+      <c r="I23" s="43">
+        <v>416</v>
+      </c>
+      <c r="J23" s="43">
+        <v>-351</v>
+      </c>
+      <c r="K23" s="43">
+        <v>-6</v>
+      </c>
+      <c r="L23" s="43">
+        <v>-357</v>
+      </c>
+      <c r="M23" s="44">
+        <f>L23/F23</f>
+        <v>0.3606060606060606</v>
+      </c>
+      <c r="N23" s="43">
+        <v>-132</v>
+      </c>
+      <c r="O23" s="43">
+        <v>191</v>
+      </c>
+      <c r="P23" s="43">
+        <f t="shared" ref="P23:P25" si="42">O23+N23</f>
+        <v>59</v>
+      </c>
+      <c r="Q23" s="45">
+        <f t="shared" ref="Q23:Q25" si="43">N23*0.11761</f>
+        <v>-15.524520000000001</v>
+      </c>
+      <c r="R23" s="45">
+        <f t="shared" ref="R23:R25" si="44">O23*0.14296</f>
+        <v>27.30536</v>
+      </c>
+      <c r="S23" s="45">
+        <f t="shared" ref="S23:S25" si="45">R23+Q23</f>
+        <v>11.78084</v>
+      </c>
+      <c r="T23" s="45">
+        <f>N23*0.01</f>
+        <v>-1.32</v>
+      </c>
+      <c r="U23" s="18">
+        <f t="shared" ref="U23:U25" si="46">(ABS(Q23)+ABS(R23))/(ABS(N23)+ABS(O23))</f>
+        <v>0.13260024767801859</v>
+      </c>
+      <c r="V23" s="19">
+        <f t="shared" ref="V23:V25" si="47">ABS(R23)/ABS(O23)</f>
+        <v>0.14296</v>
+      </c>
+      <c r="W23" s="19">
+        <f t="shared" ref="W23:W25" si="48">Q23/N23</f>
+        <v>0.11761000000000001</v>
+      </c>
+      <c r="X23" s="20">
+        <v>0.02</v>
+      </c>
+      <c r="Y23" s="20">
+        <f>Q23+R23+T23+X23</f>
+        <v>10.480839999999999</v>
+      </c>
+      <c r="Z23" s="21">
+        <v>152.74</v>
+      </c>
+      <c r="AA23" s="21">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="45">
+        <v>27.92</v>
+      </c>
+      <c r="AC23" s="45">
+        <v>-5.97</v>
+      </c>
+      <c r="AD23" s="45">
+        <v>3.43</v>
+      </c>
+      <c r="AE23" s="20">
+        <f t="shared" ref="AE23:AE25" si="49">AD23+AC23+AB23</f>
+        <v>25.380000000000003</v>
+      </c>
+      <c r="AF23" s="45">
+        <v>10</v>
+      </c>
+      <c r="AG23" s="45">
+        <v>11.36</v>
+      </c>
+      <c r="AH23" s="45">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="45">
+        <f t="shared" ref="AI23:AI25" si="50">AF23+AG23+AH23</f>
+        <v>21.36</v>
+      </c>
+      <c r="AJ23" s="46">
+        <v>0</v>
+      </c>
+      <c r="AK23" s="22">
+        <f>AA23+AI23+AJ23</f>
+        <v>21.36</v>
+      </c>
+      <c r="AL23" s="43">
+        <v>487</v>
+      </c>
+      <c r="AM23" s="43">
+        <v>168</v>
+      </c>
+      <c r="AN23" s="43">
+        <v>655</v>
+      </c>
+      <c r="AO23" s="43">
+        <v>-622</v>
+      </c>
+      <c r="AP23" s="43">
+        <v>-11</v>
+      </c>
+      <c r="AQ23" s="43">
+        <v>-633</v>
+      </c>
+      <c r="AR23" s="44">
+        <f>AQ23/F23</f>
+        <v>0.6393939393939394</v>
+      </c>
+      <c r="AS23" s="43">
+        <v>-135</v>
+      </c>
+      <c r="AT23" s="43">
+        <v>157</v>
+      </c>
+      <c r="AU23" s="43">
+        <f t="shared" ref="AU23:AU25" si="51">AT23+AS23</f>
+        <v>22</v>
+      </c>
+      <c r="AV23" s="45">
+        <f t="shared" ref="AV23:AV25" si="52">AS23*0.11761</f>
+        <v>-15.877350000000002</v>
+      </c>
+      <c r="AW23" s="45">
+        <f t="shared" ref="AW23:AW25" si="53">AT23*0.14296</f>
+        <v>22.44472</v>
+      </c>
+      <c r="AX23" s="45">
+        <f t="shared" ref="AX23:AX25" si="54">AW23+AV23</f>
+        <v>6.5673699999999986</v>
+      </c>
+      <c r="AY23" s="45">
+        <f>AS23*0.01</f>
+        <v>-1.35</v>
+      </c>
+      <c r="AZ23" s="45">
+        <v>0.01</v>
+      </c>
+      <c r="BA23" s="20">
+        <f t="shared" ref="BA23:BA25" si="55">AZ23+AY23+AX23</f>
+        <v>5.2273699999999987</v>
+      </c>
+      <c r="BB23" s="21">
+        <v>199.49</v>
+      </c>
+      <c r="BC23" s="21">
+        <v>0</v>
+      </c>
+      <c r="BD23" s="20">
+        <v>11.36</v>
+      </c>
+      <c r="BE23" s="45">
+        <v>0</v>
+      </c>
+      <c r="BF23" s="22">
+        <f t="shared" ref="BF23:BF25" si="56">BD23+BC23+BE23</f>
+        <v>11.36</v>
+      </c>
     </row>
     <row r="24" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="40"/>
-      <c r="C24" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="25">
-        <f>ROUND(J24/M22,0)</f>
-        <v>-215</v>
-      </c>
-      <c r="E24" s="25">
-        <f>ROUND(K24/M22,0)</f>
-        <v>-11</v>
-      </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25">
-        <v>62</v>
-      </c>
-      <c r="H24" s="25">
-        <v>65</v>
-      </c>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25">
-        <v>-60</v>
-      </c>
-      <c r="K24" s="25">
-        <v>-3</v>
-      </c>
-      <c r="L24" s="25"/>
-      <c r="M24" s="26"/>
-      <c r="N24" s="25"/>
-      <c r="O24" s="25"/>
-      <c r="P24" s="25"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
-      <c r="V24" s="27"/>
-      <c r="W24" s="27"/>
-      <c r="X24" s="27"/>
-      <c r="Y24" s="27"/>
-      <c r="Z24" s="27"/>
-      <c r="AA24" s="27"/>
-      <c r="AB24" s="27"/>
-      <c r="AC24" s="27"/>
-      <c r="AD24" s="27"/>
-      <c r="AE24" s="27"/>
-      <c r="AF24" s="27"/>
-      <c r="AG24" s="27"/>
-      <c r="AH24" s="27"/>
-      <c r="AI24" s="27"/>
-      <c r="AJ24" s="41"/>
-      <c r="AK24" s="27"/>
-      <c r="AL24" s="25"/>
-      <c r="AM24" s="25"/>
-      <c r="AN24" s="25"/>
-      <c r="AO24" s="25"/>
-      <c r="AP24" s="25"/>
-      <c r="AQ24" s="25"/>
-      <c r="AR24" s="26"/>
-      <c r="AS24" s="25"/>
-      <c r="AT24" s="25"/>
-      <c r="AU24" s="25"/>
-      <c r="AV24" s="27"/>
-      <c r="AW24" s="27"/>
-      <c r="AX24" s="27"/>
-      <c r="AY24" s="27"/>
-      <c r="AZ24" s="27"/>
-      <c r="BA24" s="27"/>
-      <c r="BB24" s="27"/>
-      <c r="BC24" s="27"/>
-      <c r="BD24" s="27"/>
-      <c r="BE24" s="27"/>
-      <c r="BF24" s="27"/>
+      <c r="A24" s="2"/>
+      <c r="B24" s="13">
+        <v>45631</v>
+      </c>
+      <c r="C24" s="13">
+        <v>45643</v>
+      </c>
+      <c r="D24" s="15">
+        <f>ROUND(J24/M24,0)</f>
+        <v>-605</v>
+      </c>
+      <c r="E24" s="15">
+        <f t="shared" ref="E24:E25" si="57">ROUND(K24/M24,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="15">
+        <v>-605</v>
+      </c>
+      <c r="G24" s="15">
+        <v>350</v>
+      </c>
+      <c r="H24" s="15">
+        <v>214</v>
+      </c>
+      <c r="I24" s="15">
+        <v>564</v>
+      </c>
+      <c r="J24" s="15">
+        <v>-206</v>
+      </c>
+      <c r="K24" s="15">
+        <v>0</v>
+      </c>
+      <c r="L24" s="15">
+        <v>-206</v>
+      </c>
+      <c r="M24" s="16">
+        <f t="shared" ref="M24" si="58">L24/F24</f>
+        <v>0.34049586776859503</v>
+      </c>
+      <c r="N24" s="15">
+        <v>144</v>
+      </c>
+      <c r="O24" s="15">
+        <v>214</v>
+      </c>
+      <c r="P24" s="15">
+        <f t="shared" si="42"/>
+        <v>358</v>
+      </c>
+      <c r="Q24" s="17">
+        <f t="shared" si="43"/>
+        <v>16.935840000000002</v>
+      </c>
+      <c r="R24" s="17">
+        <f t="shared" si="44"/>
+        <v>30.593440000000001</v>
+      </c>
+      <c r="S24" s="17">
+        <f t="shared" si="45"/>
+        <v>47.52928</v>
+      </c>
+      <c r="T24" s="17">
+        <v>0</v>
+      </c>
+      <c r="U24" s="18">
+        <f t="shared" si="46"/>
+        <v>0.13276335195530725</v>
+      </c>
+      <c r="V24" s="19">
+        <f t="shared" si="47"/>
+        <v>0.14296</v>
+      </c>
+      <c r="W24" s="19">
+        <f t="shared" si="48"/>
+        <v>0.11761000000000002</v>
+      </c>
+      <c r="X24" s="20">
+        <v>0.02</v>
+      </c>
+      <c r="Y24" s="20">
+        <f>Q24+R24+T24+X24</f>
+        <v>47.549280000000003</v>
+      </c>
+      <c r="Z24" s="21">
+        <v>105.1</v>
+      </c>
+      <c r="AA24" s="21">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="17">
+        <v>120.14</v>
+      </c>
+      <c r="AC24" s="17">
+        <v>-36.22</v>
+      </c>
+      <c r="AD24" s="17">
+        <v>8.11</v>
+      </c>
+      <c r="AE24" s="20">
+        <f t="shared" si="49"/>
+        <v>92.03</v>
+      </c>
+      <c r="AF24" s="17">
+        <v>10</v>
+      </c>
+      <c r="AG24" s="17">
+        <v>12.14</v>
+      </c>
+      <c r="AH24" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI24" s="17">
+        <f t="shared" si="50"/>
+        <v>22.14</v>
+      </c>
+      <c r="AJ24" s="47">
+        <v>0</v>
+      </c>
+      <c r="AK24" s="22">
+        <f>AA24+AI24+AJ24</f>
+        <v>22.14</v>
+      </c>
+      <c r="AL24" s="15">
+        <f t="shared" ref="AL24:AM24" si="59">AS24-AO24</f>
+        <v>599</v>
+      </c>
+      <c r="AM24" s="15">
+        <f t="shared" si="59"/>
+        <v>242</v>
+      </c>
+      <c r="AN24" s="15">
+        <v>841</v>
+      </c>
+      <c r="AO24" s="15">
+        <f>D24-J24</f>
+        <v>-399</v>
+      </c>
+      <c r="AP24" s="15">
+        <f>E24-K24</f>
+        <v>0</v>
+      </c>
+      <c r="AQ24" s="15">
+        <v>-399</v>
+      </c>
+      <c r="AR24" s="16">
+        <f>AQ24/F24</f>
+        <v>0.65950413223140492</v>
+      </c>
+      <c r="AS24" s="15">
+        <v>200</v>
+      </c>
+      <c r="AT24" s="15">
+        <v>242</v>
+      </c>
+      <c r="AU24" s="15">
+        <f t="shared" si="51"/>
+        <v>442</v>
+      </c>
+      <c r="AV24" s="17">
+        <f t="shared" si="52"/>
+        <v>23.522000000000002</v>
+      </c>
+      <c r="AW24" s="17">
+        <f t="shared" si="53"/>
+        <v>34.596319999999999</v>
+      </c>
+      <c r="AX24" s="17">
+        <f t="shared" si="54"/>
+        <v>58.118319999999997</v>
+      </c>
+      <c r="AY24" s="17">
+        <v>0</v>
+      </c>
+      <c r="AZ24" s="17">
+        <v>0.13</v>
+      </c>
+      <c r="BA24" s="20">
+        <f t="shared" si="55"/>
+        <v>58.24832</v>
+      </c>
+      <c r="BB24" s="21">
+        <v>141.24</v>
+      </c>
+      <c r="BC24" s="21">
+        <v>0</v>
+      </c>
+      <c r="BD24" s="20">
+        <v>12.14</v>
+      </c>
+      <c r="BE24" s="17">
+        <v>0</v>
+      </c>
+      <c r="BF24" s="22">
+        <f t="shared" si="56"/>
+        <v>12.14</v>
+      </c>
     </row>
     <row r="25" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="7"/>
-      <c r="B25" s="42">
-        <v>45600</v>
-      </c>
-      <c r="C25" s="42">
-        <v>45610</v>
-      </c>
-      <c r="D25" s="43">
-        <f>ROUND(J25/M25,0)</f>
-        <v>-973</v>
-      </c>
-      <c r="E25" s="43">
-        <f>ROUND(K25/M25,0)</f>
-        <v>-17</v>
-      </c>
-      <c r="F25" s="43">
-        <v>-990</v>
-      </c>
-      <c r="G25" s="43">
-        <v>219</v>
-      </c>
-      <c r="H25" s="43">
-        <v>197</v>
-      </c>
-      <c r="I25" s="43">
-        <v>416</v>
-      </c>
-      <c r="J25" s="43">
-        <v>-351</v>
-      </c>
-      <c r="K25" s="43">
-        <v>-6</v>
-      </c>
-      <c r="L25" s="43">
-        <v>-357</v>
-      </c>
-      <c r="M25" s="44">
+      <c r="A25" s="2"/>
+      <c r="B25" s="13">
+        <v>45663</v>
+      </c>
+      <c r="C25" s="13">
+        <v>45673</v>
+      </c>
+      <c r="D25" s="15">
+        <f t="shared" ref="D25" si="60">ROUND(J25/M25,0)</f>
+        <v>-309</v>
+      </c>
+      <c r="E25" s="15">
+        <f t="shared" si="57"/>
+        <v>0</v>
+      </c>
+      <c r="F25" s="15">
+        <v>-309</v>
+      </c>
+      <c r="G25" s="15">
+        <f t="shared" ref="G25:H25" si="61">G26+G27</f>
+        <v>489</v>
+      </c>
+      <c r="H25" s="15">
+        <f t="shared" si="61"/>
+        <v>332</v>
+      </c>
+      <c r="I25" s="15">
+        <v>821</v>
+      </c>
+      <c r="J25" s="15">
+        <f t="shared" ref="J25:K25" si="62">J26+J27</f>
+        <v>-210</v>
+      </c>
+      <c r="K25" s="15">
+        <f t="shared" si="62"/>
+        <v>0</v>
+      </c>
+      <c r="L25" s="15">
+        <v>-210</v>
+      </c>
+      <c r="M25" s="16">
         <f>L25/F25</f>
-        <v>0.3606060606060606</v>
-      </c>
-      <c r="N25" s="43">
-        <v>-132</v>
-      </c>
-      <c r="O25" s="43">
-        <v>191</v>
-      </c>
-      <c r="P25" s="43">
-        <f t="shared" ref="P25:P27" si="45">O25+N25</f>
-        <v>59</v>
-      </c>
-      <c r="Q25" s="45">
-        <f t="shared" ref="Q25:Q27" si="46">N25*0.11761</f>
-        <v>-15.524520000000001</v>
-      </c>
-      <c r="R25" s="45">
-        <f t="shared" ref="R25:R27" si="47">O25*0.14296</f>
-        <v>27.30536</v>
-      </c>
-      <c r="S25" s="45">
-        <f t="shared" ref="S25:S27" si="48">R25+Q25</f>
-        <v>11.78084</v>
-      </c>
-      <c r="T25" s="45">
-        <f>N25*0.01</f>
-        <v>-1.32</v>
+        <v>0.67961165048543692</v>
+      </c>
+      <c r="N25" s="15">
+        <v>279</v>
+      </c>
+      <c r="O25" s="15">
+        <v>332</v>
+      </c>
+      <c r="P25" s="15">
+        <f t="shared" si="42"/>
+        <v>611</v>
+      </c>
+      <c r="Q25" s="17">
+        <f t="shared" si="43"/>
+        <v>32.813189999999999</v>
+      </c>
+      <c r="R25" s="17">
+        <f t="shared" si="44"/>
+        <v>47.462720000000004</v>
+      </c>
+      <c r="S25" s="17">
+        <f t="shared" si="45"/>
+        <v>80.27591000000001</v>
+      </c>
+      <c r="T25" s="17">
+        <v>0</v>
       </c>
       <c r="U25" s="18">
-        <f t="shared" ref="U25:U27" si="49">(ABS(Q25)+ABS(R25))/(ABS(N25)+ABS(O25))</f>
-        <v>0.13260024767801859</v>
+        <f t="shared" si="46"/>
+        <v>0.1313844680851064</v>
       </c>
       <c r="V25" s="19">
-        <f t="shared" ref="V25:V27" si="50">ABS(R25)/ABS(O25)</f>
+        <f t="shared" si="47"/>
         <v>0.14296</v>
       </c>
       <c r="W25" s="19">
-        <f t="shared" ref="W25:W27" si="51">Q25/N25</f>
-        <v>0.11761000000000001</v>
+        <f t="shared" si="48"/>
+        <v>0.11760999999999999</v>
       </c>
       <c r="X25" s="20">
-        <v>0.02</v>
+        <v>0.18</v>
       </c>
       <c r="Y25" s="20">
         <f>Q25+R25+T25+X25</f>
-        <v>10.480839999999999</v>
+        <v>80.455910000000017</v>
       </c>
       <c r="Z25" s="21">
-        <v>152.74</v>
+        <v>24.65</v>
       </c>
       <c r="AA25" s="21">
         <v>0</v>
       </c>
-      <c r="AB25" s="45">
-        <v>27.92</v>
-      </c>
-      <c r="AC25" s="45">
-        <v>-5.97</v>
-      </c>
-      <c r="AD25" s="45">
-        <v>3.43</v>
+      <c r="AB25" s="17">
+        <v>201.73</v>
+      </c>
+      <c r="AC25" s="17">
+        <v>-41.77</v>
+      </c>
+      <c r="AD25" s="17">
+        <v>12.56</v>
       </c>
       <c r="AE25" s="20">
-        <f t="shared" ref="AE25:AE27" si="52">AD25+AC25+AB25</f>
-        <v>25.380000000000003</v>
-      </c>
-      <c r="AF25" s="45">
+        <f t="shared" si="49"/>
+        <v>172.51999999999998</v>
+      </c>
+      <c r="AF25" s="17">
         <v>10</v>
       </c>
-      <c r="AG25" s="45">
-        <v>11.36</v>
-      </c>
-      <c r="AH25" s="45">
-        <v>0</v>
-      </c>
-      <c r="AI25" s="45">
-        <f t="shared" ref="AI25:AI27" si="53">AF25+AG25+AH25</f>
-        <v>21.36</v>
-      </c>
-      <c r="AJ25" s="46">
+      <c r="AG25" s="17">
+        <v>12.53</v>
+      </c>
+      <c r="AH25" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI25" s="17">
+        <f t="shared" si="50"/>
+        <v>22.53</v>
+      </c>
+      <c r="AJ25" s="47">
         <v>0</v>
       </c>
       <c r="AK25" s="22">
         <f>AA25+AI25+AJ25</f>
-        <v>21.36</v>
-      </c>
-      <c r="AL25" s="43">
-        <v>487</v>
-      </c>
-      <c r="AM25" s="43">
-        <v>168</v>
-      </c>
-      <c r="AN25" s="43">
-        <v>655</v>
-      </c>
-      <c r="AO25" s="43">
-        <v>-622</v>
-      </c>
-      <c r="AP25" s="43">
-        <v>-11</v>
-      </c>
-      <c r="AQ25" s="43">
-        <v>-633</v>
-      </c>
-      <c r="AR25" s="44">
+        <v>22.53</v>
+      </c>
+      <c r="AL25" s="15">
+        <f t="shared" ref="AL25:AM25" si="63">AS25-AO25</f>
+        <v>693</v>
+      </c>
+      <c r="AM25" s="15">
+        <f t="shared" si="63"/>
+        <v>231</v>
+      </c>
+      <c r="AN25" s="15">
+        <v>924</v>
+      </c>
+      <c r="AO25" s="15">
+        <f>D25-J25</f>
+        <v>-99</v>
+      </c>
+      <c r="AP25" s="15">
+        <f>E25-K25</f>
+        <v>0</v>
+      </c>
+      <c r="AQ25" s="15">
+        <v>-99</v>
+      </c>
+      <c r="AR25" s="16">
         <f>AQ25/F25</f>
-        <v>0.6393939393939394</v>
-      </c>
-      <c r="AS25" s="43">
-        <v>-135</v>
-      </c>
-      <c r="AT25" s="43">
-        <v>157</v>
-      </c>
-      <c r="AU25" s="43">
-        <f t="shared" ref="AU25:AU27" si="54">AT25+AS25</f>
-        <v>22</v>
-      </c>
-      <c r="AV25" s="45">
-        <f t="shared" ref="AV25:AV27" si="55">AS25*0.11761</f>
-        <v>-15.877350000000002</v>
-      </c>
-      <c r="AW25" s="45">
-        <f t="shared" ref="AW25:AW27" si="56">AT25*0.14296</f>
-        <v>22.44472</v>
-      </c>
-      <c r="AX25" s="45">
-        <f t="shared" ref="AX25:AX27" si="57">AW25+AV25</f>
-        <v>6.5673699999999986</v>
-      </c>
-      <c r="AY25" s="45">
-        <f>AS25*0.01</f>
-        <v>-1.35</v>
-      </c>
-      <c r="AZ25" s="45">
-        <v>0.01</v>
+        <v>0.32038834951456313</v>
+      </c>
+      <c r="AS25" s="15">
+        <v>594</v>
+      </c>
+      <c r="AT25" s="15">
+        <v>231</v>
+      </c>
+      <c r="AU25" s="15">
+        <f t="shared" si="51"/>
+        <v>825</v>
+      </c>
+      <c r="AV25" s="17">
+        <f t="shared" si="52"/>
+        <v>69.860340000000008</v>
+      </c>
+      <c r="AW25" s="17">
+        <f t="shared" si="53"/>
+        <v>33.023760000000003</v>
+      </c>
+      <c r="AX25" s="17">
+        <f t="shared" si="54"/>
+        <v>102.88410000000002</v>
+      </c>
+      <c r="AY25" s="17">
+        <v>0</v>
+      </c>
+      <c r="AZ25" s="17">
+        <v>0.25</v>
       </c>
       <c r="BA25" s="20">
-        <f t="shared" ref="BA25:BA27" si="58">AZ25+AY25+AX25</f>
-        <v>5.2273699999999987</v>
+        <f t="shared" si="55"/>
+        <v>103.13410000000002</v>
       </c>
       <c r="BB25" s="21">
-        <v>199.49</v>
+        <v>38.11</v>
       </c>
       <c r="BC25" s="21">
         <v>0</v>
       </c>
       <c r="BD25" s="20">
-        <v>11.36</v>
-      </c>
-      <c r="BE25" s="45">
+        <v>12.53</v>
+      </c>
+      <c r="BE25" s="17">
         <v>0</v>
       </c>
       <c r="BF25" s="22">
-        <f t="shared" ref="BF25:BF27" si="59">BD25+BC25+BE25</f>
-        <v>11.36</v>
+        <f t="shared" si="56"/>
+        <v>12.53</v>
       </c>
     </row>
     <row r="26" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="2"/>
-      <c r="B26" s="13">
-        <v>45631</v>
-      </c>
-      <c r="C26" s="13">
-        <v>45643</v>
-      </c>
-      <c r="D26" s="15">
-        <f>ROUND(J26/M26,0)</f>
-        <v>-605</v>
-      </c>
-      <c r="E26" s="15">
-        <f t="shared" ref="E26:E27" si="60">ROUND(K26/M26,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F26" s="15">
-        <v>-605</v>
-      </c>
-      <c r="G26" s="15">
-        <v>350</v>
-      </c>
-      <c r="H26" s="15">
-        <v>214</v>
-      </c>
-      <c r="I26" s="15">
-        <v>564</v>
-      </c>
-      <c r="J26" s="15">
-        <v>-206</v>
-      </c>
-      <c r="K26" s="15">
-        <v>0</v>
-      </c>
-      <c r="L26" s="15">
-        <v>-206</v>
-      </c>
-      <c r="M26" s="16">
-        <f t="shared" ref="M26" si="61">L26/F26</f>
-        <v>0.34049586776859503</v>
-      </c>
-      <c r="N26" s="15">
-        <v>144</v>
-      </c>
-      <c r="O26" s="15">
-        <v>214</v>
-      </c>
-      <c r="P26" s="15">
-        <f t="shared" si="45"/>
-        <v>358</v>
-      </c>
-      <c r="Q26" s="17">
-        <f t="shared" si="46"/>
-        <v>16.935840000000002</v>
-      </c>
-      <c r="R26" s="17">
-        <f t="shared" si="47"/>
-        <v>30.593440000000001</v>
-      </c>
-      <c r="S26" s="17">
-        <f t="shared" si="48"/>
-        <v>47.52928</v>
-      </c>
-      <c r="T26" s="17">
-        <v>0</v>
-      </c>
-      <c r="U26" s="18">
-        <f t="shared" si="49"/>
-        <v>0.13276335195530725</v>
-      </c>
-      <c r="V26" s="19">
-        <f t="shared" si="50"/>
-        <v>0.14296</v>
-      </c>
-      <c r="W26" s="19">
-        <f t="shared" si="51"/>
-        <v>0.11761000000000002</v>
-      </c>
-      <c r="X26" s="20">
-        <v>0.02</v>
-      </c>
-      <c r="Y26" s="20">
-        <f>Q26+R26+T26+X26</f>
-        <v>47.549280000000003</v>
-      </c>
-      <c r="Z26" s="21">
-        <v>105.1</v>
-      </c>
-      <c r="AA26" s="21">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="17">
-        <v>120.14</v>
-      </c>
-      <c r="AC26" s="17">
-        <v>-36.22</v>
-      </c>
-      <c r="AD26" s="17">
-        <v>8.11</v>
-      </c>
-      <c r="AE26" s="20">
-        <f t="shared" si="52"/>
-        <v>92.03</v>
-      </c>
-      <c r="AF26" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG26" s="17">
-        <v>12.14</v>
-      </c>
-      <c r="AH26" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI26" s="17">
-        <f t="shared" si="53"/>
-        <v>22.14</v>
-      </c>
-      <c r="AJ26" s="47">
-        <v>0</v>
-      </c>
-      <c r="AK26" s="22">
-        <f>AA26+AI26+AJ26</f>
-        <v>22.14</v>
-      </c>
-      <c r="AL26" s="15">
-        <f t="shared" ref="AL26:AM26" si="62">AS26-AO26</f>
-        <v>599</v>
-      </c>
-      <c r="AM26" s="15">
-        <f t="shared" si="62"/>
-        <v>242</v>
-      </c>
-      <c r="AN26" s="15">
-        <v>841</v>
-      </c>
-      <c r="AO26" s="15">
-        <f>D26-J26</f>
-        <v>-399</v>
-      </c>
-      <c r="AP26" s="15">
-        <f>E26-K26</f>
-        <v>0</v>
-      </c>
-      <c r="AQ26" s="15">
-        <v>-399</v>
-      </c>
-      <c r="AR26" s="16">
-        <f>AQ26/F26</f>
-        <v>0.65950413223140492</v>
-      </c>
-      <c r="AS26" s="15">
-        <v>200</v>
-      </c>
-      <c r="AT26" s="15">
-        <v>242</v>
-      </c>
-      <c r="AU26" s="15">
-        <f t="shared" si="54"/>
-        <v>442</v>
-      </c>
-      <c r="AV26" s="17">
-        <f t="shared" si="55"/>
-        <v>23.522000000000002</v>
-      </c>
-      <c r="AW26" s="17">
-        <f t="shared" si="56"/>
-        <v>34.596319999999999</v>
-      </c>
-      <c r="AX26" s="17">
-        <f t="shared" si="57"/>
-        <v>58.118319999999997</v>
-      </c>
-      <c r="AY26" s="17">
-        <v>0</v>
-      </c>
-      <c r="AZ26" s="17">
-        <v>0.13</v>
-      </c>
-      <c r="BA26" s="20">
-        <f t="shared" si="58"/>
-        <v>58.24832</v>
-      </c>
-      <c r="BB26" s="21">
-        <v>141.24</v>
-      </c>
-      <c r="BC26" s="21">
-        <v>0</v>
-      </c>
-      <c r="BD26" s="20">
-        <v>12.14</v>
-      </c>
-      <c r="BE26" s="17">
-        <v>0</v>
-      </c>
-      <c r="BF26" s="22">
-        <f t="shared" si="59"/>
-        <v>12.14</v>
-      </c>
+      <c r="A26" s="4"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="36">
+        <f>ROUND(J26/M25,0)</f>
+        <v>-283</v>
+      </c>
+      <c r="E26" s="36">
+        <f>ROUND(K26/M25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29">
+        <v>370</v>
+      </c>
+      <c r="H26" s="29">
+        <v>241</v>
+      </c>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29">
+        <v>-192</v>
+      </c>
+      <c r="K26" s="29">
+        <v>0</v>
+      </c>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
+      <c r="O26" s="29"/>
+      <c r="P26" s="29"/>
+      <c r="Q26" s="32"/>
+      <c r="R26" s="32"/>
+      <c r="S26" s="32"/>
+      <c r="T26" s="32"/>
+      <c r="U26" s="32"/>
+      <c r="V26" s="32"/>
+      <c r="W26" s="32"/>
+      <c r="X26" s="32"/>
+      <c r="Y26" s="32"/>
+      <c r="Z26" s="32"/>
+      <c r="AA26" s="32"/>
+      <c r="AB26" s="32"/>
+      <c r="AC26" s="32"/>
+      <c r="AD26" s="32"/>
+      <c r="AE26" s="32"/>
+      <c r="AF26" s="32"/>
+      <c r="AG26" s="32"/>
+      <c r="AH26" s="32"/>
+      <c r="AI26" s="32"/>
+      <c r="AJ26" s="48"/>
+      <c r="AK26" s="32"/>
+      <c r="AL26" s="29"/>
+      <c r="AM26" s="29"/>
+      <c r="AN26" s="29"/>
+      <c r="AO26" s="29"/>
+      <c r="AP26" s="29"/>
+      <c r="AQ26" s="29"/>
+      <c r="AR26" s="30"/>
+      <c r="AS26" s="29"/>
+      <c r="AT26" s="29"/>
+      <c r="AU26" s="29"/>
+      <c r="AV26" s="32"/>
+      <c r="AW26" s="32"/>
+      <c r="AX26" s="32"/>
+      <c r="AY26" s="32"/>
+      <c r="AZ26" s="32"/>
+      <c r="BA26" s="32"/>
+      <c r="BB26" s="32"/>
+      <c r="BC26" s="32"/>
+      <c r="BD26" s="32"/>
+      <c r="BE26" s="32"/>
+      <c r="BF26" s="32"/>
     </row>
     <row r="27" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="13">
-        <v>45663</v>
-      </c>
-      <c r="C27" s="13">
-        <v>45673</v>
-      </c>
-      <c r="D27" s="15">
-        <f t="shared" ref="D27" si="63">ROUND(J27/M27,0)</f>
-        <v>-309</v>
-      </c>
-      <c r="E27" s="15">
-        <f t="shared" si="60"/>
-        <v>0</v>
-      </c>
-      <c r="F27" s="15">
-        <v>-309</v>
-      </c>
-      <c r="G27" s="15">
-        <f t="shared" ref="G27:H27" si="64">G28+G29</f>
-        <v>489</v>
-      </c>
-      <c r="H27" s="15">
-        <f t="shared" si="64"/>
-        <v>332</v>
-      </c>
-      <c r="I27" s="15">
-        <v>821</v>
-      </c>
-      <c r="J27" s="15">
-        <f t="shared" ref="J27:K27" si="65">J28+J29</f>
-        <v>-210</v>
-      </c>
-      <c r="K27" s="15">
-        <f t="shared" si="65"/>
-        <v>0</v>
-      </c>
-      <c r="L27" s="15">
-        <v>-210</v>
-      </c>
-      <c r="M27" s="16">
-        <f>L27/F27</f>
-        <v>0.67961165048543692</v>
-      </c>
-      <c r="N27" s="15">
-        <v>279</v>
-      </c>
-      <c r="O27" s="15">
-        <v>332</v>
-      </c>
-      <c r="P27" s="15">
-        <f t="shared" si="45"/>
-        <v>611</v>
-      </c>
-      <c r="Q27" s="17">
-        <f t="shared" si="46"/>
-        <v>32.813189999999999</v>
-      </c>
-      <c r="R27" s="17">
-        <f t="shared" si="47"/>
-        <v>47.462720000000004</v>
-      </c>
-      <c r="S27" s="17">
-        <f t="shared" si="48"/>
-        <v>80.27591000000001</v>
-      </c>
-      <c r="T27" s="17">
-        <v>0</v>
-      </c>
-      <c r="U27" s="18">
-        <f t="shared" si="49"/>
-        <v>0.1313844680851064</v>
-      </c>
-      <c r="V27" s="19">
-        <f t="shared" si="50"/>
-        <v>0.14296</v>
-      </c>
-      <c r="W27" s="19">
-        <f t="shared" si="51"/>
-        <v>0.11760999999999999</v>
-      </c>
-      <c r="X27" s="20">
-        <v>0.18</v>
-      </c>
-      <c r="Y27" s="20">
-        <f>Q27+R27+T27+X27</f>
-        <v>80.455910000000017</v>
-      </c>
-      <c r="Z27" s="21">
-        <v>24.65</v>
-      </c>
-      <c r="AA27" s="21">
-        <v>0</v>
-      </c>
-      <c r="AB27" s="17">
-        <v>201.73</v>
-      </c>
-      <c r="AC27" s="17">
-        <v>-41.77</v>
-      </c>
-      <c r="AD27" s="17">
-        <v>12.56</v>
-      </c>
-      <c r="AE27" s="20">
-        <f t="shared" si="52"/>
-        <v>172.51999999999998</v>
-      </c>
-      <c r="AF27" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG27" s="17">
-        <v>12.53</v>
-      </c>
-      <c r="AH27" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI27" s="17">
-        <f t="shared" si="53"/>
-        <v>22.53</v>
-      </c>
-      <c r="AJ27" s="47">
-        <v>0</v>
-      </c>
-      <c r="AK27" s="22">
-        <f>AA27+AI27+AJ27</f>
-        <v>22.53</v>
-      </c>
-      <c r="AL27" s="15">
-        <f t="shared" ref="AL27:AM27" si="66">AS27-AO27</f>
-        <v>693</v>
-      </c>
-      <c r="AM27" s="15">
-        <f t="shared" si="66"/>
-        <v>231</v>
-      </c>
-      <c r="AN27" s="15">
-        <v>924</v>
-      </c>
-      <c r="AO27" s="15">
-        <f>D27-J27</f>
-        <v>-99</v>
-      </c>
-      <c r="AP27" s="15">
-        <f>E27-K27</f>
-        <v>0</v>
-      </c>
-      <c r="AQ27" s="15">
-        <v>-99</v>
-      </c>
-      <c r="AR27" s="16">
-        <f>AQ27/F27</f>
-        <v>0.32038834951456313</v>
-      </c>
-      <c r="AS27" s="15">
-        <v>594</v>
-      </c>
-      <c r="AT27" s="15">
-        <v>231</v>
-      </c>
-      <c r="AU27" s="15">
-        <f t="shared" si="54"/>
-        <v>825</v>
-      </c>
-      <c r="AV27" s="17">
-        <f t="shared" si="55"/>
-        <v>69.860340000000008</v>
-      </c>
-      <c r="AW27" s="17">
-        <f t="shared" si="56"/>
-        <v>33.023760000000003</v>
-      </c>
-      <c r="AX27" s="17">
-        <f t="shared" si="57"/>
-        <v>102.88410000000002</v>
-      </c>
-      <c r="AY27" s="17">
-        <v>0</v>
-      </c>
-      <c r="AZ27" s="17">
-        <v>0.25</v>
-      </c>
-      <c r="BA27" s="20">
-        <f t="shared" si="58"/>
-        <v>103.13410000000002</v>
-      </c>
-      <c r="BB27" s="21">
-        <v>38.11</v>
-      </c>
-      <c r="BC27" s="21">
-        <v>0</v>
-      </c>
-      <c r="BD27" s="20">
-        <v>12.53</v>
-      </c>
-      <c r="BE27" s="17">
-        <v>0</v>
-      </c>
-      <c r="BF27" s="22">
-        <f t="shared" si="59"/>
-        <v>12.53</v>
-      </c>
+      <c r="A27" s="4"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="36">
+        <f>ROUND(J27/M25,0)</f>
+        <v>-26</v>
+      </c>
+      <c r="E27" s="36">
+        <f>ROUND(K27/M25,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29">
+        <v>119</v>
+      </c>
+      <c r="H27" s="29">
+        <v>91</v>
+      </c>
+      <c r="I27" s="29"/>
+      <c r="J27" s="29">
+        <v>-18</v>
+      </c>
+      <c r="K27" s="29">
+        <v>0</v>
+      </c>
+      <c r="L27" s="29"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="29"/>
+      <c r="O27" s="29"/>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="32"/>
+      <c r="R27" s="32"/>
+      <c r="S27" s="32"/>
+      <c r="T27" s="32"/>
+      <c r="U27" s="32"/>
+      <c r="V27" s="32"/>
+      <c r="W27" s="32"/>
+      <c r="X27" s="32"/>
+      <c r="Y27" s="32"/>
+      <c r="Z27" s="32"/>
+      <c r="AA27" s="32"/>
+      <c r="AB27" s="32"/>
+      <c r="AC27" s="32"/>
+      <c r="AD27" s="32"/>
+      <c r="AE27" s="32"/>
+      <c r="AF27" s="32"/>
+      <c r="AG27" s="32"/>
+      <c r="AH27" s="32"/>
+      <c r="AI27" s="32"/>
+      <c r="AJ27" s="48"/>
+      <c r="AK27" s="32"/>
+      <c r="AL27" s="29"/>
+      <c r="AM27" s="29"/>
+      <c r="AN27" s="29"/>
+      <c r="AO27" s="29"/>
+      <c r="AP27" s="29"/>
+      <c r="AQ27" s="29"/>
+      <c r="AR27" s="30"/>
+      <c r="AS27" s="29"/>
+      <c r="AT27" s="29"/>
+      <c r="AU27" s="29"/>
+      <c r="AV27" s="32"/>
+      <c r="AW27" s="32"/>
+      <c r="AX27" s="32"/>
+      <c r="AY27" s="32"/>
+      <c r="AZ27" s="32"/>
+      <c r="BA27" s="32"/>
+      <c r="BB27" s="32"/>
+      <c r="BC27" s="32"/>
+      <c r="BD27" s="32"/>
+      <c r="BE27" s="32"/>
+      <c r="BF27" s="32"/>
     </row>
     <row r="28" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="36">
-        <f>ROUND(J28/M27,0)</f>
-        <v>-283</v>
-      </c>
-      <c r="E28" s="36">
-        <f>ROUND(K28/M27,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29">
-        <v>370</v>
-      </c>
-      <c r="H28" s="29">
-        <v>241</v>
-      </c>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29">
-        <v>-192</v>
-      </c>
-      <c r="K28" s="29">
-        <v>0</v>
-      </c>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="29"/>
-      <c r="O28" s="29"/>
-      <c r="P28" s="29"/>
-      <c r="Q28" s="32"/>
-      <c r="R28" s="32"/>
-      <c r="S28" s="32"/>
-      <c r="T28" s="32"/>
-      <c r="U28" s="32"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="32"/>
-      <c r="X28" s="32"/>
-      <c r="Y28" s="32"/>
-      <c r="Z28" s="32"/>
-      <c r="AA28" s="32"/>
-      <c r="AB28" s="32"/>
-      <c r="AC28" s="32"/>
-      <c r="AD28" s="32"/>
-      <c r="AE28" s="32"/>
-      <c r="AF28" s="32"/>
-      <c r="AG28" s="32"/>
-      <c r="AH28" s="32"/>
-      <c r="AI28" s="32"/>
-      <c r="AJ28" s="48"/>
-      <c r="AK28" s="32"/>
-      <c r="AL28" s="29"/>
-      <c r="AM28" s="29"/>
-      <c r="AN28" s="29"/>
-      <c r="AO28" s="29"/>
-      <c r="AP28" s="29"/>
-      <c r="AQ28" s="29"/>
-      <c r="AR28" s="30"/>
-      <c r="AS28" s="29"/>
-      <c r="AT28" s="29"/>
-      <c r="AU28" s="29"/>
-      <c r="AV28" s="32"/>
-      <c r="AW28" s="32"/>
-      <c r="AX28" s="32"/>
-      <c r="AY28" s="32"/>
-      <c r="AZ28" s="32"/>
-      <c r="BA28" s="32"/>
-      <c r="BB28" s="32"/>
-      <c r="BC28" s="32"/>
-      <c r="BD28" s="32"/>
-      <c r="BE28" s="32"/>
-      <c r="BF28" s="32"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="13">
+        <v>45692</v>
+      </c>
+      <c r="C28" s="13">
+        <v>45707</v>
+      </c>
+      <c r="D28" s="15">
+        <v>0</v>
+      </c>
+      <c r="E28" s="15">
+        <v>0</v>
+      </c>
+      <c r="F28" s="15">
+        <v>0</v>
+      </c>
+      <c r="G28" s="15">
+        <v>615</v>
+      </c>
+      <c r="H28" s="15">
+        <v>332</v>
+      </c>
+      <c r="I28" s="15">
+        <f>G28+H28</f>
+        <v>947</v>
+      </c>
+      <c r="J28" s="15">
+        <v>0</v>
+      </c>
+      <c r="K28" s="15">
+        <v>-190</v>
+      </c>
+      <c r="L28" s="15">
+        <v>-190</v>
+      </c>
+      <c r="M28" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="N28" s="15">
+        <v>615</v>
+      </c>
+      <c r="O28" s="15">
+        <v>142</v>
+      </c>
+      <c r="P28" s="15">
+        <v>757</v>
+      </c>
+      <c r="Q28" s="17">
+        <v>72.33</v>
+      </c>
+      <c r="R28" s="17">
+        <v>20.3</v>
+      </c>
+      <c r="S28" s="17">
+        <f>R28+Q28</f>
+        <v>92.63</v>
+      </c>
+      <c r="T28" s="17">
+        <v>-10</v>
+      </c>
+      <c r="U28" s="18">
+        <f t="shared" ref="U28:U29" si="64">(ABS(Q28)+ABS(R28))/(ABS(N28)+ABS(O28))</f>
+        <v>0.12236459709379127</v>
+      </c>
+      <c r="V28" s="19">
+        <f t="shared" ref="V28:V29" si="65">ABS(R28)/ABS(O28)</f>
+        <v>0.14295774647887324</v>
+      </c>
+      <c r="W28" s="19">
+        <f t="shared" ref="W28:W29" si="66">Q28/N28</f>
+        <v>0.11760975609756097</v>
+      </c>
+      <c r="X28" s="20">
+        <v>0</v>
+      </c>
+      <c r="Y28" s="20">
+        <f>Q28+R28+T28+X28</f>
+        <v>82.63</v>
+      </c>
+      <c r="Z28" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="21">
+        <f>Y28-14.65+0.23</f>
+        <v>68.209999999999994</v>
+      </c>
+      <c r="AB28" s="17">
+        <v>248.1</v>
+      </c>
+      <c r="AC28" s="17">
+        <v>-37.92</v>
+      </c>
+      <c r="AD28" s="17">
+        <v>14.16</v>
+      </c>
+      <c r="AE28" s="20">
+        <f>AD28+AC28+AB28</f>
+        <v>224.34</v>
+      </c>
+      <c r="AF28" s="17">
+        <v>10</v>
+      </c>
+      <c r="AG28" s="17">
+        <v>11.36</v>
+      </c>
+      <c r="AH28" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI28" s="17">
+        <f t="shared" ref="AI28:AI29" si="67">AF28+AG28+AH28</f>
+        <v>21.36</v>
+      </c>
+      <c r="AJ28" s="47">
+        <v>0</v>
+      </c>
+      <c r="AK28" s="22">
+        <f>AA28+AI28+AJ28</f>
+        <v>89.57</v>
+      </c>
+      <c r="AL28" s="15">
+        <f t="shared" ref="AL28:AM28" si="68">AS28-AO28</f>
+        <v>732</v>
+      </c>
+      <c r="AM28" s="15">
+        <f t="shared" si="68"/>
+        <v>9</v>
+      </c>
+      <c r="AN28" s="15">
+        <v>741</v>
+      </c>
+      <c r="AO28" s="15">
+        <f t="shared" ref="AO28:AP31" si="69">D28-J28</f>
+        <v>0</v>
+      </c>
+      <c r="AP28" s="15">
+        <f t="shared" si="69"/>
+        <v>190</v>
+      </c>
+      <c r="AQ28" s="15">
+        <v>190</v>
+      </c>
+      <c r="AR28" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="AS28" s="15">
+        <v>732</v>
+      </c>
+      <c r="AT28" s="15">
+        <v>199</v>
+      </c>
+      <c r="AU28" s="15">
+        <f t="shared" ref="AU28:AU30" si="70">AT28+AS28</f>
+        <v>931</v>
+      </c>
+      <c r="AV28" s="17">
+        <f>AS28*0.11761</f>
+        <v>86.090519999999998</v>
+      </c>
+      <c r="AW28" s="17">
+        <f>AT28*0.14296</f>
+        <v>28.44904</v>
+      </c>
+      <c r="AX28" s="17">
+        <f t="shared" ref="AX28:AX29" si="71">AW28+AV28</f>
+        <v>114.53955999999999</v>
+      </c>
+      <c r="AY28" s="17">
+        <v>0</v>
+      </c>
+      <c r="AZ28" s="17">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="BA28" s="20">
+        <f t="shared" ref="BA28:BA29" si="72">AZ28+AY28+AX28</f>
+        <v>114.81956</v>
+      </c>
+      <c r="BB28" s="21">
+        <v>0</v>
+      </c>
+      <c r="BC28" s="21">
+        <v>76.709999999999994</v>
+      </c>
+      <c r="BD28" s="20">
+        <v>11.36</v>
+      </c>
+      <c r="BE28" s="17">
+        <v>0</v>
+      </c>
+      <c r="BF28" s="22">
+        <f t="shared" ref="BF28:BF29" si="73">BD28+BC28+BE28</f>
+        <v>88.07</v>
+      </c>
     </row>
     <row r="29" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="4"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="D29" s="36">
-        <f>ROUND(J29/M27,0)</f>
-        <v>-26</v>
-      </c>
-      <c r="E29" s="36">
-        <f>ROUND(K29/M27,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29">
-        <v>119</v>
-      </c>
-      <c r="H29" s="29">
-        <v>91</v>
-      </c>
-      <c r="I29" s="29"/>
-      <c r="J29" s="29">
-        <v>-18</v>
-      </c>
-      <c r="K29" s="29">
-        <v>0</v>
-      </c>
-      <c r="L29" s="29"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="29"/>
-      <c r="O29" s="29"/>
-      <c r="P29" s="29"/>
-      <c r="Q29" s="32"/>
-      <c r="R29" s="32"/>
-      <c r="S29" s="32"/>
-      <c r="T29" s="32"/>
-      <c r="U29" s="32"/>
-      <c r="V29" s="32"/>
-      <c r="W29" s="32"/>
-      <c r="X29" s="32"/>
-      <c r="Y29" s="32"/>
-      <c r="Z29" s="32"/>
-      <c r="AA29" s="32"/>
-      <c r="AB29" s="32"/>
-      <c r="AC29" s="32"/>
-      <c r="AD29" s="32"/>
-      <c r="AE29" s="32"/>
-      <c r="AF29" s="32"/>
-      <c r="AG29" s="32"/>
-      <c r="AH29" s="32"/>
-      <c r="AI29" s="32"/>
-      <c r="AJ29" s="48"/>
-      <c r="AK29" s="32"/>
-      <c r="AL29" s="29"/>
-      <c r="AM29" s="29"/>
-      <c r="AN29" s="29"/>
-      <c r="AO29" s="29"/>
-      <c r="AP29" s="29"/>
-      <c r="AQ29" s="29"/>
-      <c r="AR29" s="30"/>
-      <c r="AS29" s="29"/>
-      <c r="AT29" s="29"/>
-      <c r="AU29" s="29"/>
-      <c r="AV29" s="32"/>
-      <c r="AW29" s="32"/>
-      <c r="AX29" s="32"/>
-      <c r="AY29" s="32"/>
-      <c r="AZ29" s="32"/>
-      <c r="BA29" s="32"/>
-      <c r="BB29" s="32"/>
-      <c r="BC29" s="32"/>
-      <c r="BD29" s="32"/>
-      <c r="BE29" s="32"/>
-      <c r="BF29" s="32"/>
+      <c r="A29" s="2"/>
+      <c r="B29" s="13">
+        <v>45722</v>
+      </c>
+      <c r="C29" s="13">
+        <v>45730</v>
+      </c>
+      <c r="D29" s="15">
+        <f>ROUND(J29/M29,0)</f>
+        <v>-760</v>
+      </c>
+      <c r="E29" s="15">
+        <f>ROUND(K29/M29,0)</f>
+        <v>-2</v>
+      </c>
+      <c r="F29" s="15">
+        <v>-762</v>
+      </c>
+      <c r="G29" s="15">
+        <f t="shared" ref="G29:H29" si="74">G30+G31</f>
+        <v>321</v>
+      </c>
+      <c r="H29" s="15">
+        <f t="shared" si="74"/>
+        <v>286</v>
+      </c>
+      <c r="I29" s="15">
+        <v>607</v>
+      </c>
+      <c r="J29" s="15">
+        <f t="shared" ref="J29:K29" si="75">J30+J31</f>
+        <v>-304</v>
+      </c>
+      <c r="K29" s="15">
+        <f t="shared" si="75"/>
+        <v>-1</v>
+      </c>
+      <c r="L29" s="15">
+        <v>-305</v>
+      </c>
+      <c r="M29" s="16">
+        <f>L29/F29</f>
+        <v>0.40026246719160102</v>
+      </c>
+      <c r="N29" s="15">
+        <v>17</v>
+      </c>
+      <c r="O29" s="15">
+        <v>285</v>
+      </c>
+      <c r="P29" s="15">
+        <v>302</v>
+      </c>
+      <c r="Q29" s="17">
+        <f t="shared" ref="Q29:S29" si="76">Q30+Q31</f>
+        <v>1.9100000000000001</v>
+      </c>
+      <c r="R29" s="17">
+        <f t="shared" si="76"/>
+        <v>38.949999999999996</v>
+      </c>
+      <c r="S29" s="17">
+        <f t="shared" si="76"/>
+        <v>40.859999999999992</v>
+      </c>
+      <c r="T29" s="17">
+        <v>0</v>
+      </c>
+      <c r="U29" s="18">
+        <f t="shared" si="64"/>
+        <v>0.1352980132450331</v>
+      </c>
+      <c r="V29" s="19">
+        <f t="shared" si="65"/>
+        <v>0.13666666666666666</v>
+      </c>
+      <c r="W29" s="19">
+        <f t="shared" si="66"/>
+        <v>0.1123529411764706</v>
+      </c>
+      <c r="X29" s="20">
+        <v>0.09</v>
+      </c>
+      <c r="Y29" s="20">
+        <f>Q29+R29+T29+X29</f>
+        <v>40.950000000000003</v>
+      </c>
+      <c r="Z29" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="21">
+        <v>40.950000000000003</v>
+      </c>
+      <c r="AB29" s="17">
+        <v>106.04</v>
+      </c>
+      <c r="AC29" s="17">
+        <v>-30.72</v>
+      </c>
+      <c r="AD29" s="17">
+        <v>6.77</v>
+      </c>
+      <c r="AE29" s="20">
+        <v>82.09</v>
+      </c>
+      <c r="AF29" s="17">
+        <v>10</v>
+      </c>
+      <c r="AG29" s="17">
+        <v>11.82</v>
+      </c>
+      <c r="AH29" s="17">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="17">
+        <f t="shared" si="67"/>
+        <v>21.82</v>
+      </c>
+      <c r="AJ29" s="15">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="22">
+        <f>AA29+AI29+AJ29</f>
+        <v>62.77</v>
+      </c>
+      <c r="AL29" s="15">
+        <f t="shared" ref="AL29:AM29" si="77">AS29-AO29</f>
+        <v>592</v>
+      </c>
+      <c r="AM29" s="15">
+        <f t="shared" si="77"/>
+        <v>242</v>
+      </c>
+      <c r="AN29" s="15">
+        <v>834</v>
+      </c>
+      <c r="AO29" s="15">
+        <f t="shared" si="69"/>
+        <v>-456</v>
+      </c>
+      <c r="AP29" s="15">
+        <f t="shared" si="69"/>
+        <v>-1</v>
+      </c>
+      <c r="AQ29" s="15">
+        <v>-457</v>
+      </c>
+      <c r="AR29" s="16">
+        <f>AQ29/F29</f>
+        <v>0.59973753280839892</v>
+      </c>
+      <c r="AS29" s="15">
+        <f t="shared" ref="AS29:AT29" si="78">AS30+AS31</f>
+        <v>136</v>
+      </c>
+      <c r="AT29" s="15">
+        <f t="shared" si="78"/>
+        <v>241</v>
+      </c>
+      <c r="AU29" s="15">
+        <f t="shared" si="70"/>
+        <v>377</v>
+      </c>
+      <c r="AV29" s="17">
+        <f t="shared" ref="AV29:AW29" si="79">AV30+AV31</f>
+        <v>15.293426873</v>
+      </c>
+      <c r="AW29" s="17">
+        <f t="shared" si="79"/>
+        <v>32.941085250999997</v>
+      </c>
+      <c r="AX29" s="17">
+        <f t="shared" si="71"/>
+        <v>48.234512123999998</v>
+      </c>
+      <c r="AY29" s="17">
+        <v>0</v>
+      </c>
+      <c r="AZ29" s="17">
+        <v>0.11</v>
+      </c>
+      <c r="BA29" s="20">
+        <f t="shared" si="72"/>
+        <v>48.344512123999998</v>
+      </c>
+      <c r="BB29" s="21">
+        <v>0</v>
+      </c>
+      <c r="BC29" s="21">
+        <f>BA29</f>
+        <v>48.344512123999998</v>
+      </c>
+      <c r="BD29" s="20">
+        <v>11.82</v>
+      </c>
+      <c r="BE29" s="17">
+        <v>0</v>
+      </c>
+      <c r="BF29" s="22">
+        <f t="shared" si="73"/>
+        <v>60.164512123999998</v>
+      </c>
     </row>
     <row r="30" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="2"/>
-      <c r="B30" s="13">
-        <v>45692</v>
-      </c>
-      <c r="C30" s="13">
-        <v>45707</v>
-      </c>
-      <c r="D30" s="15">
-        <v>0</v>
-      </c>
-      <c r="E30" s="15">
-        <v>0</v>
-      </c>
-      <c r="F30" s="15">
-        <v>0</v>
-      </c>
-      <c r="G30" s="15">
-        <v>615</v>
-      </c>
-      <c r="H30" s="15">
-        <v>332</v>
-      </c>
-      <c r="I30" s="15">
-        <f>G30+H30</f>
-        <v>947</v>
-      </c>
-      <c r="J30" s="15">
-        <v>0</v>
-      </c>
-      <c r="K30" s="15">
-        <v>-190</v>
-      </c>
-      <c r="L30" s="15">
-        <v>-190</v>
-      </c>
-      <c r="M30" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="N30" s="15">
-        <v>615</v>
-      </c>
-      <c r="O30" s="15">
-        <v>142</v>
-      </c>
-      <c r="P30" s="15">
-        <v>757</v>
-      </c>
-      <c r="Q30" s="17">
-        <v>72.33</v>
-      </c>
-      <c r="R30" s="17">
-        <v>20.3</v>
-      </c>
-      <c r="S30" s="17">
-        <f>R30+Q30</f>
-        <v>92.63</v>
-      </c>
-      <c r="T30" s="17">
-        <v>-10</v>
-      </c>
-      <c r="U30" s="18">
-        <f t="shared" ref="U30:U31" si="67">(ABS(Q30)+ABS(R30))/(ABS(N30)+ABS(O30))</f>
-        <v>0.12236459709379127</v>
-      </c>
-      <c r="V30" s="19">
-        <f t="shared" ref="V30:V31" si="68">ABS(R30)/ABS(O30)</f>
-        <v>0.14295774647887324</v>
-      </c>
-      <c r="W30" s="19">
-        <f t="shared" ref="W30:W31" si="69">Q30/N30</f>
-        <v>0.11760975609756097</v>
-      </c>
-      <c r="X30" s="20">
-        <v>0</v>
-      </c>
-      <c r="Y30" s="20">
-        <f>Q30+R30+T30+X30</f>
-        <v>82.63</v>
-      </c>
-      <c r="Z30" s="21">
-        <v>0</v>
-      </c>
-      <c r="AA30" s="21">
-        <f>Y30-14.65+0.23</f>
-        <v>68.209999999999994</v>
-      </c>
-      <c r="AB30" s="17">
-        <v>248.1</v>
-      </c>
-      <c r="AC30" s="17">
-        <v>-37.92</v>
-      </c>
-      <c r="AD30" s="17">
-        <v>14.16</v>
-      </c>
-      <c r="AE30" s="20">
-        <f>AD30+AC30+AB30</f>
-        <v>224.34</v>
-      </c>
-      <c r="AF30" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG30" s="17">
-        <v>11.36</v>
-      </c>
-      <c r="AH30" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI30" s="17">
-        <f t="shared" ref="AI30:AI31" si="70">AF30+AG30+AH30</f>
-        <v>21.36</v>
-      </c>
-      <c r="AJ30" s="47">
-        <v>0</v>
-      </c>
-      <c r="AK30" s="22">
-        <f>AA30+AI30+AJ30</f>
-        <v>89.57</v>
-      </c>
-      <c r="AL30" s="15">
-        <f t="shared" ref="AL30:AM30" si="71">AS30-AO30</f>
-        <v>732</v>
-      </c>
-      <c r="AM30" s="15">
-        <f t="shared" si="71"/>
-        <v>9</v>
-      </c>
-      <c r="AN30" s="15">
-        <v>741</v>
-      </c>
-      <c r="AO30" s="15">
-        <f t="shared" ref="AO30:AP33" si="72">D30-J30</f>
-        <v>0</v>
-      </c>
-      <c r="AP30" s="15">
-        <f t="shared" si="72"/>
-        <v>190</v>
-      </c>
-      <c r="AQ30" s="15">
-        <v>190</v>
-      </c>
-      <c r="AR30" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="AS30" s="15">
-        <v>732</v>
-      </c>
-      <c r="AT30" s="15">
-        <v>199</v>
-      </c>
-      <c r="AU30" s="15">
-        <f t="shared" ref="AU30:AU32" si="73">AT30+AS30</f>
-        <v>931</v>
-      </c>
-      <c r="AV30" s="17">
-        <f>AS30*0.11761</f>
-        <v>86.090519999999998</v>
-      </c>
-      <c r="AW30" s="17">
-        <f>AT30*0.14296</f>
-        <v>28.44904</v>
-      </c>
-      <c r="AX30" s="17">
-        <f t="shared" ref="AX30:AX31" si="74">AW30+AV30</f>
-        <v>114.53955999999999</v>
-      </c>
-      <c r="AY30" s="17">
-        <v>0</v>
-      </c>
-      <c r="AZ30" s="17">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="BA30" s="20">
-        <f t="shared" ref="BA30:BA31" si="75">AZ30+AY30+AX30</f>
-        <v>114.81956</v>
-      </c>
-      <c r="BB30" s="21">
-        <v>0</v>
-      </c>
-      <c r="BC30" s="21">
-        <v>76.709999999999994</v>
-      </c>
-      <c r="BD30" s="20">
-        <v>11.36</v>
-      </c>
-      <c r="BE30" s="17">
-        <v>0</v>
-      </c>
-      <c r="BF30" s="22">
-        <f t="shared" ref="BF30:BF31" si="76">BD30+BC30+BE30</f>
-        <v>88.07</v>
-      </c>
+      <c r="A30" s="8"/>
+      <c r="B30" s="50"/>
+      <c r="C30" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="D30" s="36">
+        <f>ROUND(J30/M29,0)</f>
+        <v>-597</v>
+      </c>
+      <c r="E30" s="36">
+        <f>ROUND(K30/M29,0)</f>
+        <v>-2</v>
+      </c>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36">
+        <v>268</v>
+      </c>
+      <c r="H30" s="36">
+        <v>204</v>
+      </c>
+      <c r="I30" s="36"/>
+      <c r="J30" s="36">
+        <v>-239</v>
+      </c>
+      <c r="K30" s="36">
+        <v>-1</v>
+      </c>
+      <c r="L30" s="36"/>
+      <c r="M30" s="38"/>
+      <c r="N30" s="64">
+        <v>14.166700000000001</v>
+      </c>
+      <c r="O30" s="64">
+        <v>237.5</v>
+      </c>
+      <c r="P30" s="36"/>
+      <c r="Q30" s="39">
+        <v>1.58</v>
+      </c>
+      <c r="R30" s="39">
+        <v>32.159999999999997</v>
+      </c>
+      <c r="S30" s="39">
+        <f t="shared" ref="S30:S31" si="80">Q30+R30</f>
+        <v>33.739999999999995</v>
+      </c>
+      <c r="T30" s="36"/>
+      <c r="U30" s="36"/>
+      <c r="V30" s="36"/>
+      <c r="W30" s="36"/>
+      <c r="X30" s="36"/>
+      <c r="Y30" s="36"/>
+      <c r="Z30" s="36"/>
+      <c r="AA30" s="36"/>
+      <c r="AB30" s="39"/>
+      <c r="AC30" s="39"/>
+      <c r="AD30" s="39"/>
+      <c r="AE30" s="39"/>
+      <c r="AF30" s="36"/>
+      <c r="AG30" s="39"/>
+      <c r="AH30" s="39"/>
+      <c r="AI30" s="39"/>
+      <c r="AJ30" s="39"/>
+      <c r="AK30" s="39"/>
+      <c r="AL30" s="63">
+        <f>AS30-AO30</f>
+        <v>471.33330000000001</v>
+      </c>
+      <c r="AM30" s="63">
+        <f>AT30-AP30</f>
+        <v>201.83330000000001</v>
+      </c>
+      <c r="AN30" s="36"/>
+      <c r="AO30" s="36">
+        <f t="shared" si="69"/>
+        <v>-358</v>
+      </c>
+      <c r="AP30" s="36">
+        <f t="shared" si="69"/>
+        <v>-1</v>
+      </c>
+      <c r="AQ30" s="38"/>
+      <c r="AR30" s="38"/>
+      <c r="AS30" s="36">
+        <v>113.33329999999999</v>
+      </c>
+      <c r="AT30" s="36">
+        <v>200.83330000000001</v>
+      </c>
+      <c r="AU30" s="36">
+        <f t="shared" si="70"/>
+        <v>314.16660000000002</v>
+      </c>
+      <c r="AV30" s="39">
+        <f>AS30*0.11142</f>
+        <v>12.627596285999999</v>
+      </c>
+      <c r="AW30" s="39">
+        <f>AT30*0.13543</f>
+        <v>27.198853819</v>
+      </c>
+      <c r="AX30" s="39"/>
+      <c r="AY30" s="39"/>
+      <c r="AZ30" s="39"/>
+      <c r="BA30" s="39"/>
+      <c r="BB30" s="39"/>
+      <c r="BC30" s="39"/>
+      <c r="BD30" s="39"/>
+      <c r="BE30" s="39"/>
+      <c r="BF30" s="39"/>
     </row>
     <row r="31" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="13">
-        <v>45722</v>
-      </c>
-      <c r="C31" s="13">
-        <v>45730</v>
-      </c>
-      <c r="D31" s="15">
-        <f>ROUND(J31/M31,0)</f>
-        <v>-760</v>
-      </c>
-      <c r="E31" s="15">
-        <f>ROUND(K31/M31,0)</f>
-        <v>-2</v>
-      </c>
-      <c r="F31" s="15">
-        <v>-762</v>
-      </c>
-      <c r="G31" s="15">
-        <f t="shared" ref="G31:H31" si="77">G32+G33</f>
-        <v>321</v>
-      </c>
-      <c r="H31" s="15">
-        <f t="shared" si="77"/>
-        <v>286</v>
-      </c>
-      <c r="I31" s="15">
-        <v>607</v>
-      </c>
-      <c r="J31" s="15">
-        <f t="shared" ref="J31:K31" si="78">J32+J33</f>
-        <v>-304</v>
-      </c>
-      <c r="K31" s="15">
-        <f t="shared" si="78"/>
-        <v>-1</v>
-      </c>
-      <c r="L31" s="15">
-        <v>-305</v>
-      </c>
-      <c r="M31" s="16">
-        <f>L31/F31</f>
-        <v>0.40026246719160102</v>
-      </c>
-      <c r="N31" s="15">
-        <v>17</v>
-      </c>
-      <c r="O31" s="15">
-        <v>285</v>
-      </c>
-      <c r="P31" s="15">
-        <v>302</v>
-      </c>
-      <c r="Q31" s="17">
-        <f t="shared" ref="Q31:S31" si="79">Q32+Q33</f>
-        <v>1.9100000000000001</v>
-      </c>
-      <c r="R31" s="17">
-        <f t="shared" si="79"/>
-        <v>38.949999999999996</v>
-      </c>
-      <c r="S31" s="17">
-        <f t="shared" si="79"/>
-        <v>40.859999999999992</v>
-      </c>
-      <c r="T31" s="17">
-        <v>0</v>
-      </c>
-      <c r="U31" s="18">
-        <f t="shared" si="67"/>
-        <v>0.1352980132450331</v>
-      </c>
-      <c r="V31" s="19">
-        <f t="shared" si="68"/>
-        <v>0.13666666666666666</v>
-      </c>
-      <c r="W31" s="19">
+      <c r="A31" s="8"/>
+      <c r="B31" s="50"/>
+      <c r="C31" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="36">
+        <f>ROUND(J31/M29,0)</f>
+        <v>-162</v>
+      </c>
+      <c r="E31" s="36">
+        <f>ROUND(K31/M29,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36">
+        <v>53</v>
+      </c>
+      <c r="H31" s="36">
+        <v>82</v>
+      </c>
+      <c r="I31" s="36"/>
+      <c r="J31" s="36">
+        <v>-65</v>
+      </c>
+      <c r="K31" s="36">
+        <v>0</v>
+      </c>
+      <c r="L31" s="36"/>
+      <c r="M31" s="38"/>
+      <c r="N31" s="64">
+        <v>2.8332999999999999</v>
+      </c>
+      <c r="O31" s="64">
+        <v>47.5</v>
+      </c>
+      <c r="P31" s="36"/>
+      <c r="Q31" s="39">
+        <v>0.33</v>
+      </c>
+      <c r="R31" s="39">
+        <v>6.79</v>
+      </c>
+      <c r="S31" s="39">
+        <f t="shared" si="80"/>
+        <v>7.12</v>
+      </c>
+      <c r="T31" s="36"/>
+      <c r="U31" s="36"/>
+      <c r="V31" s="36"/>
+      <c r="W31" s="36"/>
+      <c r="X31" s="36"/>
+      <c r="Y31" s="36"/>
+      <c r="Z31" s="36"/>
+      <c r="AA31" s="36"/>
+      <c r="AB31" s="39"/>
+      <c r="AC31" s="39"/>
+      <c r="AD31" s="39"/>
+      <c r="AE31" s="36"/>
+      <c r="AF31" s="36"/>
+      <c r="AG31" s="39"/>
+      <c r="AH31" s="39"/>
+      <c r="AI31" s="39"/>
+      <c r="AJ31" s="39"/>
+      <c r="AK31" s="39"/>
+      <c r="AL31" s="63">
+        <f>AS31-AO31</f>
+        <v>119.66669999999999</v>
+      </c>
+      <c r="AM31" s="63">
+        <f>AT31-AP31</f>
+        <v>40.166699999999999</v>
+      </c>
+      <c r="AN31" s="36"/>
+      <c r="AO31" s="36">
         <f t="shared" si="69"/>
-        <v>0.1123529411764706</v>
-      </c>
-      <c r="X31" s="20">
-        <v>0.09</v>
-      </c>
-      <c r="Y31" s="20">
-        <f>Q31+R31+T31+X31</f>
-        <v>40.950000000000003</v>
-      </c>
-      <c r="Z31" s="21">
-        <v>0</v>
-      </c>
-      <c r="AA31" s="21">
-        <v>40.950000000000003</v>
-      </c>
-      <c r="AB31" s="17">
-        <v>106.04</v>
-      </c>
-      <c r="AC31" s="17">
-        <v>-30.72</v>
-      </c>
-      <c r="AD31" s="17">
-        <v>6.77</v>
-      </c>
-      <c r="AE31" s="20">
-        <v>82.09</v>
-      </c>
-      <c r="AF31" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG31" s="17">
-        <v>11.82</v>
-      </c>
-      <c r="AH31" s="17">
-        <v>0</v>
-      </c>
-      <c r="AI31" s="17">
-        <f t="shared" si="70"/>
-        <v>21.82</v>
-      </c>
-      <c r="AJ31" s="15">
-        <v>0</v>
-      </c>
-      <c r="AK31" s="22">
-        <f>AA31+AI31+AJ31</f>
-        <v>62.77</v>
-      </c>
-      <c r="AL31" s="15">
-        <f t="shared" ref="AL31:AM31" si="80">AS31-AO31</f>
-        <v>592</v>
-      </c>
-      <c r="AM31" s="15">
-        <f t="shared" si="80"/>
-        <v>242</v>
-      </c>
-      <c r="AN31" s="15">
-        <v>834</v>
-      </c>
-      <c r="AO31" s="15">
-        <f t="shared" si="72"/>
-        <v>-456</v>
-      </c>
-      <c r="AP31" s="15">
-        <f t="shared" si="72"/>
-        <v>-1</v>
-      </c>
-      <c r="AQ31" s="15">
-        <v>-457</v>
-      </c>
-      <c r="AR31" s="16">
-        <f>AQ31/F31</f>
-        <v>0.59973753280839892</v>
-      </c>
-      <c r="AS31" s="15">
-        <f t="shared" ref="AS31:AT31" si="81">AS32+AS33</f>
-        <v>136</v>
-      </c>
-      <c r="AT31" s="15">
-        <f t="shared" si="81"/>
-        <v>241</v>
-      </c>
-      <c r="AU31" s="15">
-        <f t="shared" si="73"/>
-        <v>377</v>
-      </c>
-      <c r="AV31" s="17">
-        <f t="shared" ref="AV31:AW31" si="82">AV32+AV33</f>
-        <v>15.293426873</v>
-      </c>
-      <c r="AW31" s="17">
-        <f t="shared" si="82"/>
-        <v>32.941085250999997</v>
-      </c>
-      <c r="AX31" s="17">
-        <f t="shared" si="74"/>
-        <v>48.234512123999998</v>
-      </c>
-      <c r="AY31" s="17">
-        <v>0</v>
-      </c>
-      <c r="AZ31" s="17">
-        <v>0.11</v>
-      </c>
-      <c r="BA31" s="20">
-        <f t="shared" si="75"/>
-        <v>48.344512123999998</v>
-      </c>
-      <c r="BB31" s="21">
-        <v>0</v>
-      </c>
-      <c r="BC31" s="21">
-        <f>BA31</f>
-        <v>48.344512123999998</v>
-      </c>
-      <c r="BD31" s="20">
-        <v>11.82</v>
-      </c>
-      <c r="BE31" s="17">
-        <v>0</v>
-      </c>
-      <c r="BF31" s="22">
-        <f t="shared" si="76"/>
-        <v>60.164512123999998</v>
-      </c>
+        <v>-97</v>
+      </c>
+      <c r="AP31" s="36">
+        <f t="shared" si="69"/>
+        <v>0</v>
+      </c>
+      <c r="AQ31" s="38"/>
+      <c r="AR31" s="38"/>
+      <c r="AS31" s="36">
+        <v>22.666699999999999</v>
+      </c>
+      <c r="AT31" s="36">
+        <v>40.166699999999999</v>
+      </c>
+      <c r="AU31" s="36">
+        <f>AS31+AT31</f>
+        <v>62.833399999999997</v>
+      </c>
+      <c r="AV31" s="39">
+        <f>AS31*0.11761</f>
+        <v>2.6658305869999999</v>
+      </c>
+      <c r="AW31" s="39">
+        <f>AT31*0.14296</f>
+        <v>5.7422314319999996</v>
+      </c>
+      <c r="AX31" s="39"/>
+      <c r="AY31" s="39"/>
+      <c r="AZ31" s="39"/>
+      <c r="BA31" s="39"/>
+      <c r="BB31" s="39"/>
+      <c r="BC31" s="39"/>
+      <c r="BD31" s="39"/>
+      <c r="BE31" s="39"/>
+      <c r="BF31" s="39"/>
     </row>
     <row r="32" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="8"/>
-      <c r="B32" s="50"/>
-      <c r="C32" s="36" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="36">
-        <f>ROUND(J32/M31,0)</f>
-        <v>-597</v>
-      </c>
-      <c r="E32" s="36">
-        <f>ROUND(K32/M31,0)</f>
-        <v>-2</v>
-      </c>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36">
-        <v>268</v>
-      </c>
-      <c r="H32" s="36">
-        <v>204</v>
-      </c>
-      <c r="I32" s="36"/>
-      <c r="J32" s="36">
-        <v>-239</v>
-      </c>
-      <c r="K32" s="36">
-        <v>-1</v>
-      </c>
-      <c r="L32" s="36"/>
-      <c r="M32" s="38"/>
-      <c r="N32" s="65">
-        <v>14.166700000000001</v>
-      </c>
-      <c r="O32" s="65">
-        <v>237.5</v>
-      </c>
-      <c r="P32" s="36"/>
-      <c r="Q32" s="39">
-        <v>1.58</v>
-      </c>
-      <c r="R32" s="39">
-        <v>32.159999999999997</v>
-      </c>
-      <c r="S32" s="39">
-        <f t="shared" ref="S32:S33" si="83">Q32+R32</f>
-        <v>33.739999999999995</v>
-      </c>
-      <c r="T32" s="36"/>
-      <c r="U32" s="36"/>
-      <c r="V32" s="36"/>
-      <c r="W32" s="36"/>
-      <c r="X32" s="36"/>
-      <c r="Y32" s="36"/>
-      <c r="Z32" s="36"/>
-      <c r="AA32" s="36"/>
-      <c r="AB32" s="39"/>
-      <c r="AC32" s="39"/>
-      <c r="AD32" s="39"/>
-      <c r="AE32" s="39"/>
-      <c r="AF32" s="36"/>
-      <c r="AG32" s="39"/>
-      <c r="AH32" s="39"/>
-      <c r="AI32" s="39"/>
-      <c r="AJ32" s="39"/>
-      <c r="AK32" s="39"/>
-      <c r="AL32" s="63">
-        <f>AS32-AO32</f>
-        <v>471.33330000000001</v>
-      </c>
-      <c r="AM32" s="63">
-        <f>AT32-AP32</f>
-        <v>201.83330000000001</v>
-      </c>
-      <c r="AN32" s="36"/>
-      <c r="AO32" s="36">
-        <f t="shared" si="72"/>
-        <v>-358</v>
-      </c>
-      <c r="AP32" s="36">
-        <f t="shared" si="72"/>
-        <v>-1</v>
-      </c>
-      <c r="AQ32" s="38"/>
-      <c r="AR32" s="38"/>
-      <c r="AS32" s="36">
-        <v>113.33329999999999</v>
-      </c>
-      <c r="AT32" s="36">
-        <v>200.83330000000001</v>
-      </c>
-      <c r="AU32" s="36">
-        <f t="shared" si="73"/>
-        <v>314.16660000000002</v>
-      </c>
-      <c r="AV32" s="39">
-        <f>AS32*0.11142</f>
-        <v>12.627596285999999</v>
-      </c>
-      <c r="AW32" s="39">
-        <f>AT32*0.13543</f>
-        <v>27.198853819</v>
-      </c>
-      <c r="AX32" s="39"/>
-      <c r="AY32" s="39"/>
-      <c r="AZ32" s="39"/>
-      <c r="BA32" s="39"/>
-      <c r="BB32" s="39"/>
-      <c r="BC32" s="39"/>
-      <c r="BD32" s="39"/>
-      <c r="BE32" s="39"/>
-      <c r="BF32" s="39"/>
+      <c r="A32" s="2"/>
+      <c r="B32" s="13">
+        <v>45753</v>
+      </c>
+      <c r="C32" s="13">
+        <v>45763</v>
+      </c>
+      <c r="D32" s="15">
+        <f>ROUND(J32/M32,0)</f>
+        <v>-1082</v>
+      </c>
+      <c r="E32" s="15">
+        <f>ROUND(K32/M32,0)</f>
+        <v>-97</v>
+      </c>
+      <c r="F32" s="15">
+        <v>-1179</v>
+      </c>
+      <c r="G32" s="15">
+        <v>265</v>
+      </c>
+      <c r="H32" s="15">
+        <v>213</v>
+      </c>
+      <c r="I32" s="15">
+        <f>H32+G32</f>
+        <v>478</v>
+      </c>
+      <c r="J32" s="15">
+        <v>-412</v>
+      </c>
+      <c r="K32" s="15">
+        <v>-37</v>
+      </c>
+      <c r="L32" s="15">
+        <f>K32+J32</f>
+        <v>-449</v>
+      </c>
+      <c r="M32" s="16">
+        <f>L32/F32</f>
+        <v>0.38083121289228161</v>
+      </c>
+      <c r="N32" s="15">
+        <v>-147</v>
+      </c>
+      <c r="O32" s="15">
+        <v>176</v>
+      </c>
+      <c r="P32" s="15">
+        <v>29</v>
+      </c>
+      <c r="Q32" s="17">
+        <v>-16.38</v>
+      </c>
+      <c r="R32" s="17">
+        <v>23.84</v>
+      </c>
+      <c r="S32" s="17">
+        <f>R32</f>
+        <v>23.84</v>
+      </c>
+      <c r="T32" s="17">
+        <v>-1.47</v>
+      </c>
+      <c r="U32" s="18">
+        <f>(ABS(Q32)+ABS(R32))/(ABS(N32)+ABS(O32))</f>
+        <v>0.12452012383900929</v>
+      </c>
+      <c r="V32" s="19">
+        <f>ABS(R32)/ABS(O32)</f>
+        <v>0.13545454545454547</v>
+      </c>
+      <c r="W32" s="19">
+        <f>Q32/N32</f>
+        <v>0.11142857142857142</v>
+      </c>
+      <c r="X32" s="20">
+        <v>0.18</v>
+      </c>
+      <c r="Y32" s="20">
+        <f>Q32+R32+T32+X32</f>
+        <v>6.1700000000000008</v>
+      </c>
+      <c r="Z32" s="21">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="21">
+        <v>6</v>
+      </c>
+      <c r="AB32" s="17">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="17">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="17">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="20">
+        <v>236.95</v>
+      </c>
+      <c r="AF32" s="17">
+        <v>10</v>
+      </c>
+      <c r="AG32" s="17">
+        <v>12.5</v>
+      </c>
+      <c r="AH32" s="17">
+        <v>236.95</v>
+      </c>
+      <c r="AI32" s="17">
+        <f>AF32+AG32+AH32</f>
+        <v>259.45</v>
+      </c>
+      <c r="AJ32" s="17">
+        <v>-58.23</v>
+      </c>
+      <c r="AK32" s="22">
+        <f>AA32+AI32+AJ32</f>
+        <v>207.22</v>
+      </c>
+      <c r="AL32" s="15">
+        <f t="shared" ref="AL32:AM32" si="81">AS32-AO32</f>
+        <v>582</v>
+      </c>
+      <c r="AM32" s="15">
+        <f t="shared" si="81"/>
+        <v>212</v>
+      </c>
+      <c r="AN32" s="15">
+        <v>794</v>
+      </c>
+      <c r="AO32" s="15">
+        <f t="shared" ref="AO32:AP32" si="82">D32-J32</f>
+        <v>-670</v>
+      </c>
+      <c r="AP32" s="15">
+        <f t="shared" si="82"/>
+        <v>-60</v>
+      </c>
+      <c r="AQ32" s="15">
+        <v>-730</v>
+      </c>
+      <c r="AR32" s="16">
+        <f>AQ32/F32</f>
+        <v>0.61916878710771839</v>
+      </c>
+      <c r="AS32" s="15">
+        <v>-88</v>
+      </c>
+      <c r="AT32" s="15">
+        <v>152</v>
+      </c>
+      <c r="AU32" s="15">
+        <f>AT32+AS32</f>
+        <v>64</v>
+      </c>
+      <c r="AV32" s="17">
+        <v>-9.8000000000000007</v>
+      </c>
+      <c r="AW32" s="17">
+        <v>20.59</v>
+      </c>
+      <c r="AX32" s="17">
+        <f>AW32+AV32</f>
+        <v>10.79</v>
+      </c>
+      <c r="AY32" s="17">
+        <v>-0.88</v>
+      </c>
+      <c r="AZ32" s="17">
+        <v>0.02</v>
+      </c>
+      <c r="BA32" s="20">
+        <f>AZ32+AY32+AX32</f>
+        <v>9.93</v>
+      </c>
+      <c r="BB32" s="21">
+        <v>0</v>
+      </c>
+      <c r="BC32" s="21">
+        <v>9.93</v>
+      </c>
+      <c r="BD32" s="20">
+        <v>369.51</v>
+      </c>
+      <c r="BE32" s="17">
+        <v>-58.23</v>
+      </c>
+      <c r="BF32" s="22">
+        <f>BD32+BC32+BE32</f>
+        <v>321.20999999999998</v>
+      </c>
     </row>
-    <row r="33" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="8"/>
-      <c r="B33" s="50"/>
-      <c r="C33" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" s="36">
-        <f>ROUND(J33/M31,0)</f>
-        <v>-162</v>
-      </c>
-      <c r="E33" s="36">
-        <f>ROUND(K33/M31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36">
-        <v>53</v>
-      </c>
-      <c r="H33" s="36">
-        <v>82</v>
-      </c>
-      <c r="I33" s="36"/>
-      <c r="J33" s="36">
-        <v>-65</v>
-      </c>
-      <c r="K33" s="36">
-        <v>0</v>
-      </c>
-      <c r="L33" s="36"/>
-      <c r="M33" s="38"/>
-      <c r="N33" s="65">
-        <v>2.8332999999999999</v>
-      </c>
-      <c r="O33" s="65">
-        <v>47.5</v>
-      </c>
-      <c r="P33" s="36"/>
-      <c r="Q33" s="39">
-        <v>0.33</v>
-      </c>
-      <c r="R33" s="39">
-        <v>6.79</v>
-      </c>
-      <c r="S33" s="39">
-        <f t="shared" si="83"/>
-        <v>7.12</v>
-      </c>
-      <c r="T33" s="36"/>
-      <c r="U33" s="36"/>
-      <c r="V33" s="36"/>
-      <c r="W33" s="36"/>
-      <c r="X33" s="36"/>
-      <c r="Y33" s="36"/>
-      <c r="Z33" s="36"/>
-      <c r="AA33" s="36"/>
-      <c r="AB33" s="39"/>
-      <c r="AC33" s="39"/>
-      <c r="AD33" s="39"/>
-      <c r="AE33" s="36"/>
-      <c r="AF33" s="36"/>
-      <c r="AG33" s="39"/>
-      <c r="AH33" s="39"/>
-      <c r="AI33" s="39"/>
-      <c r="AJ33" s="39"/>
-      <c r="AK33" s="39"/>
-      <c r="AL33" s="63">
-        <f>AS33-AO33</f>
-        <v>119.66669999999999</v>
-      </c>
-      <c r="AM33" s="63">
-        <f>AT33-AP33</f>
-        <v>40.166699999999999</v>
-      </c>
-      <c r="AN33" s="36"/>
-      <c r="AO33" s="36">
-        <f t="shared" si="72"/>
-        <v>-97</v>
-      </c>
-      <c r="AP33" s="36">
-        <f t="shared" si="72"/>
-        <v>0</v>
-      </c>
-      <c r="AQ33" s="38"/>
-      <c r="AR33" s="38"/>
-      <c r="AS33" s="36">
-        <v>22.666699999999999</v>
-      </c>
-      <c r="AT33" s="36">
-        <v>40.166699999999999</v>
-      </c>
-      <c r="AU33" s="36">
-        <f>AS33+AT33</f>
-        <v>62.833399999999997</v>
-      </c>
-      <c r="AV33" s="39">
-        <f>AS33*0.11761</f>
-        <v>2.6658305869999999</v>
-      </c>
-      <c r="AW33" s="39">
-        <f>AT33*0.14296</f>
-        <v>5.7422314319999996</v>
-      </c>
-      <c r="AX33" s="39"/>
-      <c r="AY33" s="39"/>
-      <c r="AZ33" s="39"/>
-      <c r="BA33" s="39"/>
-      <c r="BB33" s="39"/>
-      <c r="BC33" s="39"/>
-      <c r="BD33" s="39"/>
-      <c r="BE33" s="39"/>
-      <c r="BF33" s="39"/>
+    <row r="33" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Z33" s="9"/>
+      <c r="AE33" s="9"/>
     </row>
-    <row r="34" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="2"/>
-      <c r="B34" s="13">
-        <v>45753</v>
-      </c>
-      <c r="C34" s="13">
-        <v>45763</v>
-      </c>
-      <c r="D34" s="15">
-        <f>ROUND(J34/M34,0)</f>
-        <v>-1082</v>
-      </c>
-      <c r="E34" s="15">
-        <f>ROUND(K34/M34,0)</f>
-        <v>-97</v>
-      </c>
-      <c r="F34" s="15">
-        <v>-1179</v>
-      </c>
-      <c r="G34" s="15">
-        <v>265</v>
-      </c>
-      <c r="H34" s="15">
-        <v>213</v>
-      </c>
-      <c r="I34" s="15">
-        <f>H34+G34</f>
-        <v>478</v>
-      </c>
-      <c r="J34" s="15">
-        <v>-412</v>
-      </c>
-      <c r="K34" s="15">
-        <v>-37</v>
-      </c>
-      <c r="L34" s="15">
-        <f>K34+J34</f>
-        <v>-449</v>
-      </c>
-      <c r="M34" s="16">
-        <f>L34/F34</f>
-        <v>0.38083121289228161</v>
-      </c>
-      <c r="N34" s="15">
-        <v>-147</v>
-      </c>
-      <c r="O34" s="15">
-        <v>176</v>
-      </c>
-      <c r="P34" s="15">
-        <v>29</v>
-      </c>
-      <c r="Q34" s="17">
-        <v>-16.38</v>
-      </c>
-      <c r="R34" s="17">
-        <v>23.84</v>
-      </c>
-      <c r="S34" s="17">
-        <f>R34</f>
-        <v>23.84</v>
-      </c>
-      <c r="T34" s="17">
-        <v>-1.47</v>
-      </c>
-      <c r="U34" s="18">
-        <f>(ABS(Q34)+ABS(R34))/(ABS(N34)+ABS(O34))</f>
-        <v>0.12452012383900929</v>
-      </c>
-      <c r="V34" s="19">
-        <f>ABS(R34)/ABS(O34)</f>
-        <v>0.13545454545454547</v>
-      </c>
-      <c r="W34" s="19">
-        <f>Q34/N34</f>
-        <v>0.11142857142857142</v>
-      </c>
-      <c r="X34" s="20">
-        <v>0.18</v>
-      </c>
-      <c r="Y34" s="20">
-        <f>Q34+R34+T34+X34</f>
-        <v>6.1700000000000008</v>
-      </c>
-      <c r="Z34" s="21">
-        <v>0</v>
-      </c>
-      <c r="AA34" s="21">
-        <v>6</v>
-      </c>
-      <c r="AB34" s="17">
-        <v>0</v>
-      </c>
-      <c r="AC34" s="17">
-        <v>0</v>
-      </c>
-      <c r="AD34" s="17">
-        <v>0</v>
-      </c>
-      <c r="AE34" s="20">
-        <v>236.95</v>
-      </c>
-      <c r="AF34" s="17">
-        <v>10</v>
-      </c>
-      <c r="AG34" s="17">
-        <v>12.5</v>
-      </c>
-      <c r="AH34" s="17">
-        <v>236.95</v>
-      </c>
-      <c r="AI34" s="17">
-        <f>AF34+AG34+AH34</f>
-        <v>259.45</v>
-      </c>
-      <c r="AJ34" s="17">
-        <v>-58.23</v>
-      </c>
-      <c r="AK34" s="22">
-        <f>AA34+AI34+AJ34</f>
-        <v>207.22</v>
-      </c>
-      <c r="AL34" s="15">
-        <f t="shared" ref="AL34:AM34" si="84">AS34-AO34</f>
-        <v>582</v>
-      </c>
-      <c r="AM34" s="15">
-        <f t="shared" si="84"/>
-        <v>212</v>
-      </c>
-      <c r="AN34" s="15">
-        <v>794</v>
-      </c>
-      <c r="AO34" s="15">
-        <f t="shared" ref="AO34:AP34" si="85">D34-J34</f>
-        <v>-670</v>
-      </c>
-      <c r="AP34" s="15">
-        <f t="shared" si="85"/>
-        <v>-60</v>
-      </c>
-      <c r="AQ34" s="15">
-        <v>-730</v>
-      </c>
-      <c r="AR34" s="16">
-        <f>AQ34/F34</f>
-        <v>0.61916878710771839</v>
-      </c>
-      <c r="AS34" s="15">
-        <v>-88</v>
-      </c>
-      <c r="AT34" s="15">
-        <v>152</v>
-      </c>
-      <c r="AU34" s="15">
-        <f>AT34+AS34</f>
-        <v>64</v>
-      </c>
-      <c r="AV34" s="17">
-        <v>-9.8000000000000007</v>
-      </c>
-      <c r="AW34" s="17">
-        <v>20.59</v>
-      </c>
-      <c r="AX34" s="17">
-        <f>AW34+AV34</f>
-        <v>10.79</v>
-      </c>
-      <c r="AY34" s="17">
-        <v>-0.88</v>
-      </c>
-      <c r="AZ34" s="17">
-        <v>0.02</v>
-      </c>
-      <c r="BA34" s="20">
-        <f>AZ34+AY34+AX34</f>
-        <v>9.93</v>
-      </c>
-      <c r="BB34" s="21">
-        <v>0</v>
-      </c>
-      <c r="BC34" s="21">
-        <v>9.93</v>
-      </c>
-      <c r="BD34" s="20">
-        <v>369.51</v>
-      </c>
-      <c r="BE34" s="17">
-        <v>-58.23</v>
-      </c>
-      <c r="BF34" s="22">
-        <f>BD34+BC34+BE34</f>
-        <v>321.20999999999998</v>
-      </c>
+    <row r="34" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V34" s="9"/>
+      <c r="W34" s="9"/>
+      <c r="X34" s="9"/>
+      <c r="Y34" s="9"/>
     </row>
-    <row r="35" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="Z35" s="9"/>
-      <c r="AE35" s="9"/>
+    <row r="35" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P35" s="74"/>
+      <c r="AA35" s="10"/>
+      <c r="AB35" s="10"/>
     </row>
-    <row r="36" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="V36" s="9"/>
-      <c r="W36" s="9"/>
-      <c r="X36" s="9"/>
-      <c r="Y36" s="9"/>
+    <row r="36" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T36" s="11"/>
+      <c r="Z36" s="9"/>
+      <c r="AA36" s="12"/>
+      <c r="AB36" s="9"/>
     </row>
-    <row r="37" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="AA37" s="10"/>
-      <c r="AB37" s="10"/>
+    <row r="37" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P37" s="9"/>
+      <c r="T37" s="11"/>
+      <c r="AA37" s="12"/>
+      <c r="AB37" s="9"/>
     </row>
-    <row r="38" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="T38" s="11"/>
-      <c r="Z38" s="9"/>
-      <c r="AA38" s="12"/>
-      <c r="AB38" s="9"/>
+    <row r="38" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T39" s="11"/>
     </row>
-    <row r="39" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="P39" s="9"/>
-      <c r="T39" s="11"/>
-      <c r="AA39" s="12"/>
-      <c r="AB39" s="9"/>
+    <row r="40" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="T41" s="11"/>
+      <c r="AA41" s="9"/>
+      <c r="AB41" s="9"/>
     </row>
-    <row r="40" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="T41" s="11"/>
-    </row>
-    <row r="42" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="T43" s="11"/>
+    <row r="42" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="AA43" s="9"/>
       <c r="AB43" s="9"/>
     </row>
-    <row r="44" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="AA45" s="9"/>
-      <c r="AB45" s="9"/>
+    <row r="44" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AA44" s="9"/>
+      <c r="AB44" s="9"/>
     </row>
-    <row r="46" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="AA46" s="9"/>
-      <c r="AB46" s="9"/>
-    </row>
-    <row r="47" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="16:31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -6505,8 +6385,6 @@
     <row r="1008" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1009" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1011" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1012" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B3:C3"/>

</xml_diff>